<commit_message>
fix: corrected context in dataset
</commit_message>
<xml_diff>
--- a/data/annotation/curado_planilla.xlsx
+++ b/data/annotation/curado_planilla.xlsx
@@ -645,14 +645,10 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>curro</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Negocio turbio o arreglo deshonesto</t>
-        </is>
-      </c>
+          <t>torta</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
       <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Tomás</t>
@@ -670,7 +666,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>trabajo, empleo (España)</t>
+          <t>(la acepción de España o México)</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1233,7 @@
       <c r="T8" s="9" t="inlineStr"/>
       <c r="U8" s="9" t="inlineStr"/>
     </row>
-    <row r="9" ht="120" customHeight="1">
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>CUR-008</t>
@@ -1245,12 +1241,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>negro</t>
+          <t>morocho</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Se le adjudica la palabra negro, al ser humano que proviene, en su mayoría, de un lugar pobre, además de practicar el hurto como principal habilidad y otras, como atletismo (cuando roba y lo corren los vecinos o la yuta), salto (cuando va a robar a propiedades con paredes o rejas altas) y demás.</t>
+          <t>Persona de tez morena y/o de cabello negro o castaño oscuro.</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -1260,22 +1256,22 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>suave murmullo de tu suspirar / Como ríe la vida si tus ojos negros me quieren mirar / Y si es mío el amparo de tu risa</t>
+          <t>Duki dispara aunque Mauro dude (Dude) / Soy el niño 'el año, morocho achinado / Llevo el doble caño, flow polarizado</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>El Dia Que Me Quieras · Carlos Gardel (1934)</t>
+          <t>Hello Cotto · Duki (2017)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>es que se me hace irresistible / Recuerden no hablarle de trampa al negro más flexible (King) / La vida es una y la quiero vivi' a</t>
+          <t>¿Dónde estarán Traverso, el Cordobés y el Noy / El Pardo Augusto, Flores y el Morocho Aldao? / Así empezó mi vuelo de zorzal</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Nena · Zaramay (2018)</t>
+          <t>El Cantor de Buenos Aires · Roberto Goyeneche</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr"/>
@@ -1359,7 +1355,7 @@
       <c r="T10" s="9" t="inlineStr"/>
       <c r="U10" s="9" t="inlineStr"/>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>CUR-010</t>
@@ -1367,37 +1363,37 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>pedazo</t>
+          <t>manija</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Pene.</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Tener manija es tener ansias o entusiasmo por algo.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Soportaré los golpes y jamás me rendiré / Y aunque los sueños se me rompan en pedazos / Resistiré, resistiré</t>
+          <t>Con par de champetas yo siempre corono / 'Tamo re manija y nunca paramo' / Si pinta el after ahí nos mandamo'</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Resistiré (Versión Reggaetón) · Zulma Lobato (2009)</t>
+          <t>ALLA · EL NOBA (2022)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Y en esa calle de estío, calle perdida / Dejó un pedazo de vida y se marchó / Primero hay que saber sufrir, después amar, después partir</t>
+          <t>En una cancha o en un bar / Dando la vuelta manija me doy / Subiendo al latido de esta vibración</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Naranjo en Flor · Roberto Goyeneche</t>
+          <t>Toco y me voy · Bersuit Vergarabat (2000)</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr"/>
@@ -1420,7 +1416,7 @@
       <c r="T11" s="9" t="inlineStr"/>
       <c r="U11" s="9" t="inlineStr"/>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>CUR-011</t>
@@ -1443,22 +1439,22 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Ahora las palabras mas tristes tienen sentido para mi / Intente atravesar aquellos viejos puentes / Que destrui el día en que incendie mi vida</t>
+          <t>por sonsa, a fuerza de compasión / Como quedaste en la vía y tu viejo, un pobre tano / Era chivo con los cosos pelandrunes como vos</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Reescribir Tragedias Sobre Libros Y Llamas · Dar Sangre (2008)</t>
+          <t>Lloró Como Una Mujer · Edmundo Rivero (1967)</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Aún se animan a jugar / Unos niños viejos / Gris atardecer</t>
+          <t>Mi mamá tomando merca, todo enfrente 'e mi cara (Fiumba) / Y mi viejo después de eso me echó fuera 'e la casa / Pero si no</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Gris Atardecer · Los Visitantes (1994)</t>
+          <t>OPA · Dillom (2021)</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr"/>
@@ -1481,7 +1477,7 @@
       <c r="T12" s="9" t="inlineStr"/>
       <c r="U12" s="9" t="inlineStr"/>
     </row>
-    <row r="13" ht="45" customHeight="1">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>CUR-012</t>
@@ -1489,37 +1485,37 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>cocinar</t>
+          <t>macana</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Ponerse de acuerdo un grupo de personas a espaldas de los demás.</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Error, equivocación; cosa mal hecha.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Missy en la espalda como una espada de grill (Yeah) / Tengo la cocina cerra'íta para mí / Whats up, mina? (Yo, yo, ah) Work it, hace</t>
+          <t>De envenenarse mi hermana / No hay bochinche ni macana / Que en tu homenaje no hiciera</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>KAMIKAZE · Sofía Gabanna (2023)</t>
+          <t>Apología del Tango · Tita Merello (1969)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>reina, por eso un rey a tu lado / Una noche que te cocine, unos nachos en el cine / Pero con una palabra hace que el</t>
+          <t>Rebota en la fuente / ¡Ay, qué macana! / Se posa en su frente</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Oye Baby · Zaramay (2020)</t>
+          <t>La tortuga Uga · Flor Ansaldo (2020)</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr"/>
@@ -1664,7 +1660,7 @@
       <c r="T15" s="9" t="inlineStr"/>
       <c r="U15" s="9" t="inlineStr"/>
     </row>
-    <row r="16" ht="45" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>CUR-015</t>
@@ -1672,12 +1668,12 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>papa</t>
+          <t>mango</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Que algo es muy fácil o sencillo</t>
+          <t>Sinónimo de dinero.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -1687,16 +1683,24 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Mina que fue en otros tiempos, la más papa milonguera / Y en esas noches tangueras, fue la reina del festín</t>
+          <t>De manguero doctorao / Y que un mango descubrís / Aunque lo hayan enterrao</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>El Motivo · Roberto Goyeneche</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
+          <t>Dónde Hay Un Mango? · Tita Merello (1965)</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Cuando rajés los tamangos / Buscando este mango / Que te haga morfar</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Yira, Yira · Carlos Gardel (1930)</t>
+        </is>
+      </c>
       <c r="I16" s="9" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="9" t="inlineStr"/>
@@ -1839,7 +1843,7 @@
       <c r="T18" s="9" t="inlineStr"/>
       <c r="U18" s="9" t="inlineStr"/>
     </row>
-    <row r="19" ht="60" customHeight="1">
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>CUR-018</t>
@@ -1862,24 +1866,16 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Y yo les doy mi corazón / Bailando hasta tu aparición / Sentir que flotas junto a mí</t>
+          <t>de aquí, cuántos de ellos aún están / Ahora mírame a mí, que te la puedo bailar / Solo elígeme el beat, el resto lo hace papá</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Señorita Corazón · María Gabriela Epumer (1998)</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>del frutero de la esquina me tiran azahares / Vení, que así medio bailando y medio volando / Me saco el melón para saludarte, te regalo una</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>Balada Para un Loco · Roberto Goyeneche (1969)</t>
-        </is>
-      </c>
+          <t>Vivimos Deprisa · Sofía Gabanna (2021)</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr"/>
       <c r="I19" s="9" t="inlineStr"/>
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="9" t="inlineStr"/>
@@ -2030,37 +2026,37 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>llenar</t>
+          <t>piola</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>to bother, to tire</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Wiktionary (en inglés)</t>
+          <t>Adjetivo que califica a quien resuelve situaciones gracias a su ingenio; también algo que está bueno.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Por caminos que no traen mas que problemas / Y hacen que su corazón, se llene de pena / Él dejó sus mandamientos para cumplir</t>
+          <t>Acá no se usa chupín, se viste ancho / No te hagas el piola, si en Varela sos un pancho / Si quiero te arrebato, no compro</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Sinceridad · Rabito (1999)</t>
+          <t>PICA · EL NOBA (2022)</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Y he sabido que el “guerrero” / Que murió lleno de honor / Ni murió ni fue guerrero</t>
+          <t>Estoy de gira por el barrio y mañana tengo fecha / Pero me porto piola, así la 12 no sospecha / (Fuck, try me)</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Chorra · Edmundo Rivero (1959)</t>
+          <t>A$AP · Dillom (2019)</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr"/>
@@ -2083,7 +2079,7 @@
       <c r="T22" s="9" t="inlineStr"/>
       <c r="U22" s="9" t="inlineStr"/>
     </row>
-    <row r="23" ht="45" customHeight="1">
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
           <t>CUR-022</t>
@@ -2091,12 +2087,12 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>ojo</t>
+          <t>curro</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Termini utilizado para advertir a alguien que tenga cuidado</t>
+          <t>Situación arreglada previamente, generalmente de manera injusta y/o inmoral.</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -2106,22 +2102,22 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Puedo relajar otra vez / Y bailar cuando cierro los ojos / Pensando en vos</t>
+          <t>dealer' en lo' burro' (Uh) / Aprovechen el momento y saquen provecho al curro (Uh, uh-uh) / Ya tú sabe', canto envido (Ya lo dije con susurro)</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Puedo Sentirlo · David Lebón (1986)</t>
+          <t>Freestyle Session #14 “LOS INTOCABLES” · Zaramay (2021)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Lo que sentiría cerca de ti / Te miré a los ojos, te dije, sonriendo / "Qué chica más linda que venden aquí"</t>
+          <t>Sos cadenera, flor sin berretines / Que currás a los cuores con tu rango; / Pero el choma que aceita tus patines</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>La Chica de la Boutique · Heleno (1971)</t>
+          <t>A Buenos Aires Lunfa · Edmundo Rivero (1967)</t>
         </is>
       </c>
       <c r="I23" s="9" t="inlineStr"/>
@@ -2205,7 +2201,7 @@
       <c r="T24" s="9" t="inlineStr"/>
       <c r="U24" s="9" t="inlineStr"/>
     </row>
-    <row r="25" ht="45" customHeight="1">
+    <row r="25" ht="60" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>CUR-024</t>
@@ -2213,37 +2209,37 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>rara</t>
+          <t>guita</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Rufous-tailed plantcutter (Phytotoma rara)</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Wiktionary (en inglés)</t>
+          <t>Significa dinero, plata.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Esos tacos de donde han salido / Hay que rara te veo mi niña / Si tu madre se entera verás</t>
+          <t>Y al vivo le baten rana / La guita o el vento es / El dinero que circula</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>El tiempo pasa y se va · Carlos Javier Beltrán (1982)</t>
+          <t>Milonga Lunfarda · Edmundo Rivero (1972)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Cuando de repente, de atrás de un árbol, me aparezco yo / Mezcla rara de penúltimo linyera y de primer polizonte en el viaje a Venus</t>
+          <t>fin de mes me dan miguitas para que no me queje / Puta, yo quiero mi guita, no escuchar boludeces / Estoy tan cansado de este sentimiento</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>Balada Para un Loco · Roberto Goyeneche (1969)</t>
+          <t>Mi peor enemigo · Dillom (2024)</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr"/>
@@ -2266,7 +2262,7 @@
       <c r="T25" s="9" t="inlineStr"/>
       <c r="U25" s="9" t="inlineStr"/>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>CUR-025</t>
@@ -2274,12 +2270,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>deje</t>
+          <t>chabón</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>•Cuando una persona está muy apurada y va con prisa.</t>
+          <t>Término coloquial para referirse a un chico o una chica.</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -2289,22 +2285,22 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Que mas puedo hacer cuando deje mi vida y a cambio recibi estas heridas / Solo la muerte esconde el ultimo latido debil de mi corazón</t>
+          <t>El chorro, un vulgar ladrón / Al zonzo, llaman chabón / Y al vivo le baten rana</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Reescribir Tragedias Sobre Libros Y Llamas · Dar Sangre (2008)</t>
+          <t>Milonga Lunfarda · Edmundo Rivero (1972)</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Cuando se me cierren las salidas / Y la noche no me deje en paz / Cuando sienta miedo del silencio</t>
+          <t>Ese cuerpo compadrón, algún... / Algún oscuro chabón / Será el llamado a cargarte</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Resistiré (Versión Reggaetón) · Zulma Lobato (2009)</t>
+          <t>En un feca · Edmundo Rivero (1975)</t>
         </is>
       </c>
       <c r="I26" s="9" t="inlineStr"/>
@@ -2340,12 +2336,12 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>you know; used as a space filler, usually in the middle of a sentence, or when telling a story</t>
+          <t>Muletilla para confirmar que el interlocutor sigue el relato; equivale a «¿sabés?» o «¿entendés?».</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Wiktionary (en inglés)</t>
+          <t>definición del grupo (no figura en Wikcionario ni en diccionarioargentino.com)</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -2393,32 +2389,32 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Pieza móvil o fija, situada al final de una cañería de agua, a través de cuyos agujeros sale el agua de la ducha.</t>
+          <t>Antepuesto a un sustantivo, indica que es grande o notable: flor de susto, flor de quilombo.</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Wikcionario</t>
+          <t>definición del grupo (el sentido intensificador no figura en las tres fuentes del pipeline)</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
+          <t>te da también te quita / Que se hace la viva y está muerta la mosquita / Que parecía un duro y es un flor de mantequita</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Esa mierda · Sara Hebe (2012)</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
           <t>La luz de todos los colores, cantando / El color de una piel y de una flor / Una guitarra y tu voz</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>Estaré · Los Visitantes (1996)</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>Abre la Tierra el sonido y tu voz / Son bienvenidos tu fruto y tu flor / ¿Dónde has llegado? Ven a explorar</t>
-        </is>
-      </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>Princesa Cristal · Lito Epumer (2004)</t>
         </is>
       </c>
       <c r="I28" s="9" t="inlineStr"/>
@@ -2441,7 +2437,7 @@
       <c r="T28" s="9" t="inlineStr"/>
       <c r="U28" s="9" t="inlineStr"/>
     </row>
-    <row r="29" ht="75" customHeight="1">
+    <row r="29" ht="45" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
           <t>CUR-028</t>
@@ -2449,12 +2445,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>gorrión</t>
+          <t>quilombo</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Persona vulgar, ordinaria, sin trasendencia que cree que su existencia es algoextraordinario, cuando en realidad es un sujeto totalmente precindible para la sociedad. fem: gorriona.</t>
+          <t>Forma de decir caos, desorden, pelea, un gran problema.</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -2464,16 +2460,24 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>pianta'o, pianta'o, pianta'o / Yo miro a Buenos Aires del nido de un gorrión / Y a vos te vi tan triste; vení, volá, sentí el loco</t>
+          <t>que pega como Cotto / Soy de lo' pibes del fondo (Uh), de los adicto' al quilombo (Uh) / Mejor no ronquen con mi combo (Más na')</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Balada Para un Loco · Roberto Goyeneche (1969)</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr"/>
-      <c r="H29" s="7" t="inlineStr"/>
+          <t>Hello Cotto · Duki (2017)</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Estamos todos jugados, nada nos importa ya / Sigamos haciendo quilombo / La yuta no nos va llevar</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Los Pibes Chorros · Los Pibes Chorros (2001)</t>
+        </is>
+      </c>
       <c r="I29" s="9" t="inlineStr"/>
       <c r="J29" s="9" t="inlineStr"/>
       <c r="K29" s="9" t="inlineStr"/>
@@ -2624,37 +2628,37 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>piel</t>
+          <t>capo</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Química (cohesión o entendimiento con otras personas).</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Ser capo es ser muy bueno en algo, ser el mejor.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>el viaje a Venus / Medio melón en la cabeza, las rayas de la camisa pintadas en la piel / Dos medias suelas clavadas en los pies</t>
+          <t>quedo guapo si la ven conmigo, eh / Guapo eh, guapo, uh, sapo, soy el capo del hood / Tanto al mes, tanto flu', guapo, guapo, guapo</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Balada Para un Loco · Roberto Goyeneche (1969)</t>
+          <t>Guapo · YSY A (2018)</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>La luz de todos los colores, cantando / El color de una piel y de una flor / Una guitarra y tu voz</t>
+          <t>¡Con sentimiento! / El Ruca, el Loco Ale y Toca, el capo de la villa / Re tirado y descontrolado, un pucho loco me estoy fumando</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Estaré · Los Visitantes (1996)</t>
+          <t>Pucho Loco · Damas Gratis (2008)</t>
         </is>
       </c>
       <c r="I32" s="9" t="inlineStr"/>
@@ -2761,22 +2765,22 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>"El Feriado Nacional de la Vagancia" / Birra!!! Cumbia nena / Y a bailar con las Kumbia Queers</t>
+          <t>Acá siempre son 4:20, y estamo' de la cabeza, con simpleza / Birra barata y mala en lata, má' la planta santa esa / La que calma</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Feriado Nacional · Kumbia Queers (2010)</t>
+          <t>CANGURO · WOS (2019)</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>"El Feriado Nacional de la Vagancia" / Birra!!!!! / El lunes a la noche... me quiero matar</t>
+          <t>se hace larga tengo que remar / Si es un día de calor unas birras tomar / Pero hay algo que me atrapa y no puedo escapar</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Feriado Nacional · Kumbia Queers (2010)</t>
+          <t>Lo Peor · Kumbia Queers (2015)</t>
         </is>
       </c>
       <c r="I34" s="9" t="inlineStr"/>
@@ -2868,37 +2872,37 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>clandestino</t>
+          <t>fierro</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Prostíbulo.</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Arma de fuego.</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Esto va pa' los turro' y las gata' finas / Esta noche se pica en la clandestina / Los quiero a todos los pibe' cantina</t>
+          <t>de usar tanga (Jaja) / Pa' pelea' el Luna Park, desde que hay fierro nadie e' langa / No pode' hablar de má' cuando hay dos ase'</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Tamo Chelo · El Noba (2021)</t>
+          <t>Freestyle Session #14 “LOS INTOCABLES” · Zaramay (2021)</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Acá las guacha' nos llueven y nos mueven el totó / Esta noche se pica en la clandestina / El tranza refugiado vendiendo cocaína</t>
+          <t>La mafia a tu banda la saca del vuelo / Y listo, llevo fierro cheto y chico / Porque .9 usan los milico' (Oh)</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>KAKAROTO · El Noba</t>
+          <t>Tamo Chelo (Remix) · EL NOBA (2022)</t>
         </is>
       </c>
       <c r="I36" s="9" t="inlineStr"/>
@@ -2929,37 +2933,37 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>sonar</t>
+          <t>turro</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Fracasar, terminar mal o haber caído en graves problemas. Se aplica sobre todo a personas.</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Persona de mal proceder, de poca confianza.</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Como un hilo sin nombre / Suena un poco a mi guitarra / Tengo que aprender a volar</t>
+          <t>son más de lo mismo (Oh, oh) / Y que vos querés un turro que esté puesto pa' quererte / Y pa' sacarte de tu vida normal</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Canción Para los Días de la Vida · María Gabriela Epumer (2000)</t>
+          <t>Mamichula · Trueno (2020)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Y te sientes toda una mujer / El teléfono siempre sonando / Tú contestas hablando en secreto</t>
+          <t>Pa' eso feka' tengo repelente / Yo no soy un turro, tengo el corazón valiente, yah / Yo soy del barrio desde que nací</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>El tiempo pasa y se va · Carlos Javier Beltrán (1982)</t>
+          <t>Azul y Oro · Trueno (2020)</t>
         </is>
       </c>
       <c r="I37" s="9" t="inlineStr"/>
@@ -3056,32 +3060,32 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>polo-stick; mallet</t>
+          <t>Parte posterior elevada del calzado.</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Wiktionary (en inglés)</t>
+          <t>Wikcionario</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Esos tacos de donde han salido / Hay que rara te veo mi niña</t>
+          <t>elegante hablando, lady, no hace falta un saco / Y a ti pa' ser mujer no te hacen falta tacos / Mis negro' experimentan con el amoniaco</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>El tiempo pasa y se va · Carlos Javier Beltrán (1982)</t>
+          <t>Nena · Zaramay (2018)</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>elegante hablando, lady, no hace falta un saco / Y a ti pa' ser mujer no te hacen falta tacos / Mis negro' experimentan con el amoniaco</t>
+          <t>Salta, bitch, jumpin' and jumpin' (Jumpin'), jumpin' / Bitch, now, la quiero en tacos, compitiendo como Elvira Hancock (Uh) / Que tengo mis puta' pero quiero a</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>Nena · Zaramay (2018)</t>
+          <t>Elvira · 808God (2016)</t>
         </is>
       </c>
       <c r="I39" s="9" t="inlineStr"/>
@@ -3493,22 +3497,22 @@
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Quien no hace nada, es un fiaca / La pinta es la que destaca / Los rasgos de tu apostura</t>
+          <t>Y me pongo loco, re loco, re loco / Si pinta un mellizo ella le da hasta el piso / Se va de caravana y nunca le</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Milonga Lunfarda · Edmundo Rivero (1972)</t>
+          <t>Piloto · EL NOBA (2022)</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Los hombres de mí critican la voz / El modo de andar, la pinta, la tos / Critican si ya la línea perdí</t>
+          <t>bien ahí al ritmo. ¿Cómo e'? 'tamo acá con el Maxi, si pinta, despué' a la noche o más tarde nos cruzamo' ahí pa' pega'</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>Se Dice de Mí · Tita Merello (1955)</t>
+          <t>Freestyle Session #14 “LOS INTOCABLES” · Zaramay (2021)</t>
         </is>
       </c>
       <c r="I46" s="9" t="inlineStr"/>
@@ -3531,7 +3535,7 @@
       <c r="T46" s="9" t="inlineStr"/>
       <c r="U46" s="9" t="inlineStr"/>
     </row>
-    <row r="47" ht="30" customHeight="1">
+    <row r="47" ht="45" customHeight="1">
       <c r="A47" s="7" t="inlineStr">
         <is>
           <t>CUR-046</t>
@@ -3539,12 +3543,12 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>dormirse</t>
+          <t>junar</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Distraerse. Quedar desprevenido y dar pie a que alguien se aproveche de ello.</t>
+          <t>Sinónimo de conocer, reconocer, ser conocido.</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -3554,16 +3558,24 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>La cama es una catrera / Y apoliyar es dormirse / Rajar o piantarse es irse</t>
+          <t>re del after / Y el telo paga la vuelta, y no te juno en la del Master / Me escuchan los pibito' que andan en chapa</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Milonga Lunfarda · Edmundo Rivero (1972)</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr"/>
-      <c r="H47" s="7" t="inlineStr"/>
+          <t>Del Año · EL NOBA (2021)</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>También daba clases de hombría de bien; / Junaba de noches y de madrugadas / Piloteaba aviones y más de un beguén</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>A lo Megata · Edmundo Rivero (1982)</t>
+        </is>
+      </c>
       <c r="I47" s="9" t="inlineStr"/>
       <c r="J47" s="9" t="inlineStr"/>
       <c r="K47" s="9" t="inlineStr"/>
@@ -3645,37 +3657,37 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>mama</t>
+          <t>boliche</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Alteración física y mental que resulta de beber alcohol.</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Es el lugar donde se suele ir a bailar; en otros países se conoce como discoteca.</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Tus rebusques de mujer... / Hoy me entero que tu mama / “Noble viuda de un guerrero”</t>
+          <t>gusta cuando tú te me sigue' (Sí) / Te ponen música en el boliche y te la vive' (Uh-uh) / Cumbia con reggaetón, un perreo 'e salón</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Chorra · Edmundo Rivero (1959)</t>
+          <t>Tamo Chelo (Remix) · EL NOBA (2022)</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Y yo por la pena de tanto' lune' (Lune'; ah-ah) / Mama sólo pide que yo no fume (No fume) / No sirve de na' que en</t>
+          <t>No puedo sacarla de mi mente en toda la semana / Hace cuatro meses que yo vengo a este boliche / Para verte bailar entre la gente</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>Hello Cotto · Duki (2017)</t>
+          <t>Daniela · Kumbia Queers (2010)</t>
         </is>
       </c>
       <c r="I49" s="9" t="inlineStr"/>
@@ -4125,7 +4137,7 @@
       <c r="T56" s="9" t="inlineStr"/>
       <c r="U56" s="9" t="inlineStr"/>
     </row>
-    <row r="57" ht="60" customHeight="1">
+    <row r="57" ht="45" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
           <t>CUR-056</t>
@@ -4133,37 +4145,37 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>acá</t>
+          <t>mina</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Residuo sólido indigerible del bolo alimenticio, que se excreta a través del ano.</t>
-        </is>
-      </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Mujer, chica.</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Zaramay, negro, es mi nombre, por si van a matarme / Pero acá si somos hombres, y hacemos correr la sangre / Hablame de verdes, de billetes,</t>
+          <t>en un 'pernó' mezclo a Paris con Puente Alsina / Fuiste compadre del botón y de la mina / Y hasta comadre del gavión y la pebeta</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Freestyle Session #5 · Zaramay (2019)</t>
+          <t>El Choclo · Tita Merello (1954)</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Y no es que no la escucho por ser malcriado / Es que acá todos mienten y soy desconfiado / Que me mame el bicho, estoy malandrizado</t>
+          <t>El dolor de unas cadenas que me queman las muñecas / Y una mina que arrodilla mis arrestos de varón / Yo quiero morir conmigo</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>Hello Cotto · Duki (2017)</t>
+          <t>Como Abrazo a un Rencor · Edmundo Rivero (1967)</t>
         </is>
       </c>
       <c r="I57" s="9" t="inlineStr"/>
@@ -4186,7 +4198,7 @@
       <c r="T57" s="9" t="inlineStr"/>
       <c r="U57" s="9" t="inlineStr"/>
     </row>
-    <row r="58" ht="60" customHeight="1">
+    <row r="58" ht="45" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
           <t>CUR-057</t>
@@ -4194,12 +4206,12 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>manzana</t>
+          <t>curtir</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>1• Se usa para afirmar algo, sinónimo de la palabra 'sí'. 2• También se usa para responder con sarcasmo algo que resulta ser obvio.</t>
+          <t>Gustar de algo o alguien, tener preferencia por determinada cosa, comportamiento o hábito.</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -4209,22 +4221,22 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Lento beso al partir / Tibias manzanas / Al sol robadas</t>
+          <t>cheta con money y cocaine / Me invitan un tiro y yo que las deliro, me voy a curtir a las diez / Tengan veinte o dieciséis</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>Alas de la Mañana · Lito Epumer (2004)</t>
+          <t>Guapo · YSY A (2018)</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>a tu casa a conocer a tus parientes / Tu culo es la manzana, tu lengua es de serpiente / Tu piel es la más suave y</t>
+          <t>contando lo que yo viví (-ví) / Fuck tu film, los pi' no curtimos esa ni ahí / Pueden rimar, pa', pero no ser na' más pa'</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>Muñecas · Dillom (2024)</t>
+          <t>Crow · Acru (2018)</t>
         </is>
       </c>
       <c r="I58" s="9" t="inlineStr"/>
@@ -4308,7 +4320,7 @@
       <c r="T59" s="9" t="inlineStr"/>
       <c r="U59" s="9" t="inlineStr"/>
     </row>
-    <row r="60" ht="30" customHeight="1">
+    <row r="60" ht="45" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
         <is>
           <t>CUR-059</t>
@@ -4316,12 +4328,12 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>pintar</t>
+          <t>careta</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Alude a una situación, idea, acción o cosa oportuna.</t>
+          <t>Persona hipócrita, falsa, doble cara.</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
@@ -4331,22 +4343,22 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>En la tintorería de París / La pintaron con barniz / La plancharon en francés</t>
+          <t>Acá la que más cobra suele ser la mas barata / Y siempre hay un careta que transa con una rata / ¡Basta, pará! No quiero hacerlo</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>Manuelita La Tortuga · María Elena Walsh (1964)</t>
+          <t>Esa mierda · Sara Hebe (2012)</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Amores en canciones / Pinte muchos vagones / Por eso grabo hitones</t>
+          <t>Porque al primero que se haga el ortiba / Por pancho y careta le vamos a dar / ''Mamá Chorra, tenes razón''</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>Oro Puro · 808god (2020)</t>
+          <t>Llegamos los Pibes Chorros · Los Pibes Chorros (2002)</t>
         </is>
       </c>
       <c r="I60" s="9" t="inlineStr"/>
@@ -4499,37 +4511,37 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>rojo</t>
+          <t>remera</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Que pertenece o concierne al Club Atlético Independiente, o es hincha de este equipo argentino.</t>
-        </is>
-      </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Prenda de vestir que cubre el torso, de mangas cortas; camiseta.</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Se pierde / Tu boca tan roja / Se enciende</t>
+          <t>Usa siempre el mismo pantalón / Y una remera de los Rolling Stones, la colorada / Está buena por delante y por detrás</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>A través de todo · Francisco Bochatón</t>
+          <t>La colorada · Los Pibes Chorros (2003)</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Que eras el vestigio del futuro / Rojas y verdes luces del amor / Prestidigitan bajo un halo de rouge</t>
+          <t>De una ola que no para de crecer / Hoy su cara está en todas las remeras / Es un muerto que no para de nacer</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>Los Libros de la Buena Memoria · Lito Vitale (2006)</t>
+          <t>Murguita del sur · Bersuit Vergarabat (1998)</t>
         </is>
       </c>
       <c r="I63" s="9" t="inlineStr"/>
@@ -4743,31 +4755,39 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>quiebre</t>
+          <t>faso</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>breaking, break (action and effect of breaking)</t>
-        </is>
-      </c>
-      <c r="D67" s="7" t="inlineStr">
-        <is>
-          <t>Wiktionary (en inglés)</t>
+          <t>Sinónimo de cigarrillo, puede ser de marihuana o de tabaco indistintamente.</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Hago que parezcan más viejo' que yo / Querían que quiebre, querían que enferme / Me puse más fuerte, me puse más jefe</t>
+          <t>a dos casas de mi puntero / Por eso cuando voy a comprar faso la veo / Ella me dice: "Chico, invitáme a fumar que ese es</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>GIVENCHY · Duki (2022)</t>
-        </is>
-      </c>
-      <c r="G67" s="7" t="inlineStr"/>
-      <c r="H67" s="7" t="inlineStr"/>
+          <t>Una Vela · Intoxicados (2003)</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>El recuerdo de tu voz que me decía: / "Largá el faso, las pastillas y el alcohol" / Sin embargo, yo seguí dándole duro</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>Sentimiento villero · Los Pibes Chorros (2001)</t>
+        </is>
+      </c>
       <c r="I67" s="9" t="inlineStr"/>
       <c r="J67" s="9" t="inlineStr"/>
       <c r="K67" s="9" t="inlineStr"/>
@@ -4862,7 +4882,7 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Fumar marihuana</t>
+          <t>Delatar a una persona o hacerla objeto de burla. Una persona también puede «quemarse» a sí misma.</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
@@ -4933,22 +4953,22 @@
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>Hicimos del fuego nuestra luz / Hicimos del ruido las respuestas / Caminamos los desposeídos cargando los mantos que cubrirán sus cuerpos</t>
+          <t>Encerrado en mi cuarto y afuera llovía fuerte / Escuché un ruido fuerte y fui a fijarme / Subí a la terraza y vos estabas por tirarte,</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>Pedagogía de la venganza · Cienfuegos (2021)</t>
+          <t>Últimamente · Dillom (2024)</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Estoy sin vos / En medio de este ruido / Al pie estoy</t>
+          <t>invité a salir / Vamos a la fiesta de un amigo, hay mucho escabio y mucho ruido / Un chabón me deliró y un roscazo se comió</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>Todas las ventanas · Francisco Bochatón</t>
+          <t>Qué mala suerte! · 2 Minutos (1994)</t>
         </is>
       </c>
       <c r="I70" s="9" t="inlineStr"/>
@@ -4979,37 +4999,37 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>tristes</t>
+          <t>yuta</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Canto popular de origen indígena con acento muy melancólico.</t>
-        </is>
-      </c>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>De origen lunfardo, quiere decir policía.</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Me guarde estos recuerdos / Ahora las palabras mas tristes tienen sentido para mi / Intente atravesar aquellos viejos puentes</t>
+          <t>Se creen dueños, salgan del medio, lo digo en serio / Fuera la yuta que meten al barrio, le tira a los pibe' y le mata</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Reescribir Tragedias Sobre Libros Y Llamas · Dar Sangre (2008)</t>
+          <t>CANGURO · WOS (2019)</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Negro el pelo, los ojos verde gris / Y eran suaves sus manos, y eran sus versos tristes / Como el canto de ese violín</t>
+          <t>Descarten los tubos, empiecen a correr / La yuta esta muy cerca, no da para correr / El oficial grita, "¡Contra la pared!</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>Tal vez será tu voz · Lidia Borda (2011)</t>
+          <t>Demasiado tarde (La marcha) · 2 Minutos (1994)</t>
         </is>
       </c>
       <c r="I71" s="9" t="inlineStr"/>
@@ -5106,12 +5126,12 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Mala suerte.</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Dicho de algo, que es de alto costo, caro, de precio alto.</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
@@ -5154,7 +5174,7 @@
       <c r="T73" s="9" t="inlineStr"/>
       <c r="U73" s="9" t="inlineStr"/>
     </row>
-    <row r="74" ht="60" customHeight="1">
+    <row r="74" ht="45" customHeight="1">
       <c r="A74" s="7" t="inlineStr">
         <is>
           <t>CUR-073</t>
@@ -5162,37 +5182,37 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>naranja</t>
+          <t>pucho</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>Nada, ninguna cosa.</t>
-        </is>
-      </c>
-      <c r="D74" s="7" t="inlineStr">
-        <is>
-          <t>Wikcionario</t>
+          <t>Forma en que se les dice a los cigarrillos.</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>diccionarioargentino.com</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>maniquíes me guiñan, los semáforos me dan tres luces celestes / Y las naranjas del frutero de la esquina me tiran azahares / Vení, que así medio</t>
+          <t>(Este es el balneario de los doctores) / Ni del pucho que se fuma, ni la lámpara que cuelga / (Este es el balneario de los doctores</t>
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>Balada Para un Loco · Roberto Goyeneche (1969)</t>
+          <t>El Balneario de los Doctores Crotos · Los Piojos (1998)</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Voy a cumplir mi más oscura fantasía / Conocí una cheta con la piel naranja / Ella tomaba keta y yo tomaba blanca</t>
+          <t>Re tirado y descontrolado, un pucho loco me estoy fumando / Estoy sangrando y no tengo miedo ya de morir</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>Buenos tiempos · Dillom (2024)</t>
+          <t>Pucho Loco · Damas Gratis (2008)</t>
         </is>
       </c>
       <c r="I74" s="9" t="inlineStr"/>
@@ -5299,24 +5319,16 @@
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>Y mi compa con los ojo' re nublado' / Andamo' a todo ritmo, el trucho no se frena / Los mío' responde', compa, si hay problema'</t>
+          <t>gusta que no pregunten mucho / Que estén buscando amor pero ese amor del trucho / Que sepan que el dolor y el placer es tan efímero</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>KAKAROTO · El Noba</t>
-        </is>
-      </c>
-      <c r="G76" s="7" t="inlineStr">
-        <is>
-          <t>Los tuyo' hablan mucho, ninguno hace na' / Los mío' en un trucho no te van a perdonar / Del año, coco, del año (Del año)</t>
-        </is>
-      </c>
-      <c r="H76" s="7" t="inlineStr">
-        <is>
-          <t>Del Año · El Noba (2021)</t>
-        </is>
-      </c>
+          <t>Flores &amp; Bombones · Yesan 雪山 (2025)</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr"/>
+      <c r="H76" s="7" t="inlineStr"/>
       <c r="I76" s="9" t="inlineStr"/>
       <c r="J76" s="9" t="inlineStr"/>
       <c r="K76" s="9" t="inlineStr"/>
@@ -5764,7 +5776,7 @@
       <c r="T83" s="9" t="inlineStr"/>
       <c r="U83" s="9" t="inlineStr"/>
     </row>
-    <row r="84" ht="60" customHeight="1">
+    <row r="84" ht="45" customHeight="1">
       <c r="A84" s="7" t="inlineStr">
         <is>
           <t>CUR-083</t>
@@ -5772,12 +5784,12 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>novia</t>
+          <t>bacán</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>Persona que mantiene una relación de amor con otra, especialmente cuando tiene intención de casarse o de vivir en pareja con ella.</t>
+          <t>Persona de alto nivel de vida, muy cómoda y acomodada.</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
@@ -5787,22 +5799,22 @@
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>Pompeya y, más alla, la inundación / Tu melena de novia en el recuerdo / Y tu nombre flotando en el adios...</t>
+          <t>Del barrio la mondiola sos el más rana / Y te llaman garufa por lo bacán; / Tenés más pretensiones que bataclana</t>
         </is>
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
-          <t>Sur · Aníbal Troilo</t>
+          <t>Garufa · Tita Merello (1968)</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Vacilo con las turras, hasta abajo con el trago / Le robé la novia al cheto, ahora ando cotizado / Del año, coco, del año (Del año)</t>
+          <t>Pebeta de mi barrio, papa, papusa / Que andás paseando en auto con un bacán / Que te has cortado el pelo como se usa</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>Del Año · El Noba (2021)</t>
+          <t>Pompas · Roberto Goyeneche (1967)</t>
         </is>
       </c>
       <c r="I84" s="9" t="inlineStr"/>
@@ -6143,7 +6155,7 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>Sinónimo del mate.</t>
+          <t>Sinónimo de dólares, moneda estadounidense. Un palo verde son mil dólares.</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
@@ -6268,10 +6280,10 @@
     <dataValidation sqref="J2:J91 N2:N91 S2:S91" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elegí una opción de la lista" type="list">
       <formula1>"falso_amigo,polisemico_interno,lunfardo_sin_homonimo,espanol_general"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2 K3 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K28 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 K83 K84 K85 K86 K87 K88 K89 K90 K91 O2 O3 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O28 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O68 O69 O70 O71 O72 O73 O74 O75 O76 O77 O78 O79 O80 O81 O82 O83 O84 O85 O86 O87 O88 O89 O90 O91 T2 T3 T5 T6 T7 T8 T9 T10 T11 T12 T13 T14 T15 T17 T18 T19 T20 T21 T22 T23 T24 T25 T26 T28 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 T41 T42 T43 T44 T45 T46 T49 T50 T51 T52 T53 T54 T55 T56 T57 T58 T59 T60 T61 T62 T63 T64 T65 T66 T68 T69 T70 T71 T72 T73 T74 T75 T76 T77 T78 T79 T80 T81 T82 T83 T84 T85 T86 T87 T88 T89 T90 T91" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elegí A o B" type="list">
+    <dataValidation sqref="K2 K3 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K20 K21 K22 K23 K24 K25 K26 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K77 K78 K79 K80 K81 K82 K83 K84 K85 K86 K87 K88 K89 K90 K91 O2 O3 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O20 O21 O22 O23 O24 O25 O26 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O67 O68 O69 O70 O71 O72 O73 O74 O75 O77 O78 O79 O80 O81 O82 O83 O84 O85 O86 O87 O88 O89 O90 O91 T2 T3 T5 T6 T7 T8 T9 T10 T11 T12 T13 T14 T15 T16 T17 T18 T20 T21 T22 T23 T24 T25 T26 T28 T29 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 T41 T42 T43 T44 T45 T46 T47 T49 T50 T51 T52 T53 T54 T55 T56 T57 T58 T59 T60 T61 T62 T63 T64 T65 T66 T67 T68 T69 T70 T71 T72 T73 T74 T75 T77 T78 T79 T80 T81 T82 T83 T84 T85 T86 T87 T88 T89 T90 T91" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elegí A o B" type="list">
       <formula1>"A,B"</formula1>
     </dataValidation>
-    <dataValidation sqref="K4 K16 K27 K29 K47 K48 K67 O4 O16 O27 O29 O47 O48 O67 T4 T16 T27 T29 T47 T48 T67" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Esta fila solo tiene fragmento A" type="list">
+    <dataValidation sqref="K4 K19 K27 K48 K76 O4 O19 O27 O48 O76 T4 T19 T27 T48 T76" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Esta fila solo tiene fragmento A" type="list">
       <formula1>"A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6282,42 +6294,56 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
doc: added column of data
</commit_message>
<xml_diff>
--- a/data/annotation/curado_planilla.xlsx
+++ b/data/annotation/curado_planilla.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Anotación" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anotación" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Anotación'!$A$1:$U$91</definedName>
@@ -859,9 +859,21 @@
       <c r="J2" s="9" t="inlineStr"/>
       <c r="K2" s="9" t="inlineStr"/>
       <c r="L2" s="9" t="inlineStr"/>
-      <c r="M2" s="9" t="inlineStr"/>
-      <c r="N2" s="9" t="inlineStr"/>
-      <c r="O2" s="9" t="inlineStr"/>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P2" s="9" t="inlineStr"/>
       <c r="Q2" s="7">
         <f>IF(OR(J2="",N2=""),"",IF(J2=N2,"sí","no"))</f>
@@ -920,9 +932,21 @@
       <c r="J3" s="9" t="inlineStr"/>
       <c r="K3" s="9" t="inlineStr"/>
       <c r="L3" s="9" t="inlineStr"/>
-      <c r="M3" s="9" t="inlineStr"/>
-      <c r="N3" s="9" t="inlineStr"/>
-      <c r="O3" s="9" t="inlineStr"/>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P3" s="9" t="inlineStr"/>
       <c r="Q3" s="7">
         <f>IF(OR(J3="",N3=""),"",IF(J3=N3,"sí","no"))</f>
@@ -973,9 +997,21 @@
       <c r="J4" s="9" t="inlineStr"/>
       <c r="K4" s="9" t="inlineStr"/>
       <c r="L4" s="9" t="inlineStr"/>
-      <c r="M4" s="9" t="inlineStr"/>
-      <c r="N4" s="9" t="inlineStr"/>
-      <c r="O4" s="9" t="inlineStr"/>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P4" s="9" t="inlineStr"/>
       <c r="Q4" s="7">
         <f>IF(OR(J4="",N4=""),"",IF(J4=N4,"sí","no"))</f>
@@ -1034,9 +1070,21 @@
       <c r="J5" s="9" t="inlineStr"/>
       <c r="K5" s="9" t="inlineStr"/>
       <c r="L5" s="9" t="inlineStr"/>
-      <c r="M5" s="9" t="inlineStr"/>
-      <c r="N5" s="9" t="inlineStr"/>
-      <c r="O5" s="9" t="inlineStr"/>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P5" s="9" t="inlineStr"/>
       <c r="Q5" s="7">
         <f>IF(OR(J5="",N5=""),"",IF(J5=N5,"sí","no"))</f>
@@ -1095,10 +1143,26 @@
       <c r="J6" s="9" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
       <c r="L6" s="9" t="inlineStr"/>
-      <c r="M6" s="9" t="inlineStr"/>
-      <c r="N6" s="9" t="inlineStr"/>
-      <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Elevación redondeada y plana de la piel, grano/verruga (Esp.)</t>
+        </is>
+      </c>
       <c r="Q6" s="7">
         <f>IF(OR(J6="",N6=""),"",IF(J6=N6,"sí","no"))</f>
         <v/>
@@ -1156,9 +1220,21 @@
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
       <c r="L7" s="9" t="inlineStr"/>
-      <c r="M7" s="9" t="inlineStr"/>
-      <c r="N7" s="9" t="inlineStr"/>
-      <c r="O7" s="9" t="inlineStr"/>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P7" s="9" t="inlineStr"/>
       <c r="Q7" s="7">
         <f>IF(OR(J7="",N7=""),"",IF(J7=N7,"sí","no"))</f>
@@ -1217,9 +1293,21 @@
       <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
       <c r="L8" s="9" t="inlineStr"/>
-      <c r="M8" s="9" t="inlineStr"/>
-      <c r="N8" s="9" t="inlineStr"/>
-      <c r="O8" s="9" t="inlineStr"/>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P8" s="9" t="inlineStr"/>
       <c r="Q8" s="7">
         <f>IF(OR(J8="",N8=""),"",IF(J8=N8,"sí","no"))</f>
@@ -1278,9 +1366,21 @@
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
       <c r="L9" s="9" t="inlineStr"/>
-      <c r="M9" s="9" t="inlineStr"/>
-      <c r="N9" s="9" t="inlineStr"/>
-      <c r="O9" s="9" t="inlineStr"/>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P9" s="9" t="inlineStr"/>
       <c r="Q9" s="7">
         <f>IF(OR(J9="",N9=""),"",IF(J9=N9,"sí","no"))</f>
@@ -1339,10 +1439,26 @@
       <c r="J10" s="9" t="inlineStr"/>
       <c r="K10" s="9" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr"/>
-      <c r="M10" s="9" t="inlineStr"/>
-      <c r="N10" s="9" t="inlineStr"/>
-      <c r="O10" s="9" t="inlineStr"/>
-      <c r="P10" s="9" t="inlineStr"/>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>Panza o barriga (Méx., CR, El Salv., Guat., Hond., Nic.)</t>
+        </is>
+      </c>
       <c r="Q10" s="7">
         <f>IF(OR(J10="",N10=""),"",IF(J10=N10,"sí","no"))</f>
         <v/>
@@ -1400,9 +1516,21 @@
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr"/>
-      <c r="M11" s="9" t="inlineStr"/>
-      <c r="N11" s="9" t="inlineStr"/>
-      <c r="O11" s="9" t="inlineStr"/>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P11" s="9" t="inlineStr"/>
       <c r="Q11" s="7">
         <f>IF(OR(J11="",N11=""),"",IF(J11=N11,"sí","no"))</f>
@@ -1461,10 +1589,26 @@
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr"/>
-      <c r="M12" s="9" t="inlineStr"/>
-      <c r="N12" s="9" t="inlineStr"/>
-      <c r="O12" s="9" t="inlineStr"/>
-      <c r="P12" s="9" t="inlineStr"/>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>Mujer, persona del sexo femenino (coloq.; Bol. y Méx.)</t>
+        </is>
+      </c>
       <c r="Q12" s="7">
         <f>IF(OR(J12="",N12=""),"",IF(J12=N12,"sí","no"))</f>
         <v/>
@@ -1522,9 +1666,21 @@
       <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="9" t="inlineStr"/>
       <c r="L13" s="9" t="inlineStr"/>
-      <c r="M13" s="9" t="inlineStr"/>
-      <c r="N13" s="9" t="inlineStr"/>
-      <c r="O13" s="9" t="inlineStr"/>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P13" s="9" t="inlineStr"/>
       <c r="Q13" s="7">
         <f>IF(OR(J13="",N13=""),"",IF(J13=N13,"sí","no"))</f>
@@ -1583,10 +1739,26 @@
       <c r="J14" s="9" t="inlineStr"/>
       <c r="K14" s="9" t="inlineStr"/>
       <c r="L14" s="9" t="inlineStr"/>
-      <c r="M14" s="9" t="inlineStr"/>
-      <c r="N14" s="9" t="inlineStr"/>
-      <c r="O14" s="9" t="inlineStr"/>
-      <c r="P14" s="9" t="inlineStr"/>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P14" s="9" t="inlineStr">
+        <is>
+          <t>Colín de pan pequeño (Esp.)</t>
+        </is>
+      </c>
       <c r="Q14" s="7">
         <f>IF(OR(J14="",N14=""),"",IF(J14=N14,"sí","no"))</f>
         <v/>
@@ -1644,9 +1816,21 @@
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr"/>
       <c r="L15" s="9" t="inlineStr"/>
-      <c r="M15" s="9" t="inlineStr"/>
-      <c r="N15" s="9" t="inlineStr"/>
-      <c r="O15" s="9" t="inlineStr"/>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P15" s="9" t="inlineStr"/>
       <c r="Q15" s="7">
         <f>IF(OR(J15="",N15=""),"",IF(J15=N15,"sí","no"))</f>
@@ -1658,7 +1842,11 @@
       </c>
       <c r="S15" s="9" t="inlineStr"/>
       <c r="T15" s="9" t="inlineStr"/>
-      <c r="U15" s="9" t="inlineStr"/>
+      <c r="U15" s="9" t="inlineStr">
+        <is>
+          <t>Fragmento A usa el sentido literal (pelo canoso: "...más canas que pelos tengo en el mate"), no el rioplatense (policía/preso); por eso se eligió B.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -1705,10 +1893,26 @@
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="9" t="inlineStr"/>
       <c r="L16" s="9" t="inlineStr"/>
-      <c r="M16" s="9" t="inlineStr"/>
-      <c r="N16" s="9" t="inlineStr"/>
-      <c r="O16" s="9" t="inlineStr"/>
-      <c r="P16" s="9" t="inlineStr"/>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P16" s="9" t="inlineStr">
+        <is>
+          <t>Persona guapa, atractiva (El Salv., Méx. y Nic.)</t>
+        </is>
+      </c>
       <c r="Q16" s="7">
         <f>IF(OR(J16="",N16=""),"",IF(J16=N16,"sí","no"))</f>
         <v/>
@@ -1766,9 +1970,21 @@
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="9" t="inlineStr"/>
       <c r="L17" s="9" t="inlineStr"/>
-      <c r="M17" s="9" t="inlineStr"/>
-      <c r="N17" s="9" t="inlineStr"/>
-      <c r="O17" s="9" t="inlineStr"/>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P17" s="9" t="inlineStr"/>
       <c r="Q17" s="7">
         <f>IF(OR(J17="",N17=""),"",IF(J17=N17,"sí","no"))</f>
@@ -1827,9 +2043,21 @@
       <c r="J18" s="9" t="inlineStr"/>
       <c r="K18" s="9" t="inlineStr"/>
       <c r="L18" s="9" t="inlineStr"/>
-      <c r="M18" s="9" t="inlineStr"/>
-      <c r="N18" s="9" t="inlineStr"/>
-      <c r="O18" s="9" t="inlineStr"/>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N18" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P18" s="9" t="inlineStr"/>
       <c r="Q18" s="7">
         <f>IF(OR(J18="",N18=""),"",IF(J18=N18,"sí","no"))</f>
@@ -1880,9 +2108,21 @@
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="9" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr"/>
-      <c r="M19" s="9" t="inlineStr"/>
-      <c r="N19" s="9" t="inlineStr"/>
-      <c r="O19" s="9" t="inlineStr"/>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N19" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P19" s="9" t="inlineStr"/>
       <c r="Q19" s="7">
         <f>IF(OR(J19="",N19=""),"",IF(J19=N19,"sí","no"))</f>
@@ -1941,9 +2181,21 @@
       <c r="J20" s="9" t="inlineStr"/>
       <c r="K20" s="9" t="inlineStr"/>
       <c r="L20" s="9" t="inlineStr"/>
-      <c r="M20" s="9" t="inlineStr"/>
-      <c r="N20" s="9" t="inlineStr"/>
-      <c r="O20" s="9" t="inlineStr"/>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P20" s="9" t="inlineStr"/>
       <c r="Q20" s="7">
         <f>IF(OR(J20="",N20=""),"",IF(J20=N20,"sí","no"))</f>
@@ -2002,10 +2254,26 @@
       <c r="J21" s="9" t="inlineStr"/>
       <c r="K21" s="9" t="inlineStr"/>
       <c r="L21" s="9" t="inlineStr"/>
-      <c r="M21" s="9" t="inlineStr"/>
-      <c r="N21" s="9" t="inlineStr"/>
-      <c r="O21" s="9" t="inlineStr"/>
-      <c r="P21" s="9" t="inlineStr"/>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P21" s="9" t="inlineStr">
+        <is>
+          <t>Bonita, atractiva, interesante (adj., Méx.)</t>
+        </is>
+      </c>
       <c r="Q21" s="7">
         <f>IF(OR(J21="",N21=""),"",IF(J21=N21,"sí","no"))</f>
         <v/>
@@ -2063,9 +2331,21 @@
       <c r="J22" s="9" t="inlineStr"/>
       <c r="K22" s="9" t="inlineStr"/>
       <c r="L22" s="9" t="inlineStr"/>
-      <c r="M22" s="9" t="inlineStr"/>
-      <c r="N22" s="9" t="inlineStr"/>
-      <c r="O22" s="9" t="inlineStr"/>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P22" s="9" t="inlineStr"/>
       <c r="Q22" s="7">
         <f>IF(OR(J22="",N22=""),"",IF(J22=N22,"sí","no"))</f>
@@ -2124,10 +2404,26 @@
       <c r="J23" s="9" t="inlineStr"/>
       <c r="K23" s="9" t="inlineStr"/>
       <c r="L23" s="9" t="inlineStr"/>
-      <c r="M23" s="9" t="inlineStr"/>
-      <c r="N23" s="9" t="inlineStr"/>
-      <c r="O23" s="9" t="inlineStr"/>
-      <c r="P23" s="9" t="inlineStr"/>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P23" s="9" t="inlineStr">
+        <is>
+          <t>Trabajo o labor (uso cotidiano en España; el DLE no lo marca regionalmente)</t>
+        </is>
+      </c>
       <c r="Q23" s="7">
         <f>IF(OR(J23="",N23=""),"",IF(J23=N23,"sí","no"))</f>
         <v/>
@@ -2185,10 +2481,26 @@
       <c r="J24" s="9" t="inlineStr"/>
       <c r="K24" s="9" t="inlineStr"/>
       <c r="L24" s="9" t="inlineStr"/>
-      <c r="M24" s="9" t="inlineStr"/>
-      <c r="N24" s="9" t="inlineStr"/>
-      <c r="O24" s="9" t="inlineStr"/>
-      <c r="P24" s="9" t="inlineStr"/>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N24" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O24" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P24" s="9" t="inlineStr">
+        <is>
+          <t>Tonto, estúpido (muy asociado a México; el DLE no lo marca regionalmente)</t>
+        </is>
+      </c>
       <c r="Q24" s="7">
         <f>IF(OR(J24="",N24=""),"",IF(J24=N24,"sí","no"))</f>
         <v/>
@@ -2246,9 +2558,21 @@
       <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="9" t="inlineStr"/>
       <c r="L25" s="9" t="inlineStr"/>
-      <c r="M25" s="9" t="inlineStr"/>
-      <c r="N25" s="9" t="inlineStr"/>
-      <c r="O25" s="9" t="inlineStr"/>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N25" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O25" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P25" s="9" t="inlineStr"/>
       <c r="Q25" s="7">
         <f>IF(OR(J25="",N25=""),"",IF(J25=N25,"sí","no"))</f>
@@ -2307,9 +2631,21 @@
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="9" t="inlineStr"/>
       <c r="L26" s="9" t="inlineStr"/>
-      <c r="M26" s="9" t="inlineStr"/>
-      <c r="N26" s="9" t="inlineStr"/>
-      <c r="O26" s="9" t="inlineStr"/>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P26" s="9" t="inlineStr"/>
       <c r="Q26" s="7">
         <f>IF(OR(J26="",N26=""),"",IF(J26=N26,"sí","no"))</f>
@@ -2360,9 +2696,21 @@
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="9" t="inlineStr"/>
       <c r="L27" s="9" t="inlineStr"/>
-      <c r="M27" s="9" t="inlineStr"/>
-      <c r="N27" s="9" t="inlineStr"/>
-      <c r="O27" s="9" t="inlineStr"/>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N27" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P27" s="9" t="inlineStr"/>
       <c r="Q27" s="7">
         <f>IF(OR(J27="",N27=""),"",IF(J27=N27,"sí","no"))</f>
@@ -2374,7 +2722,11 @@
       </c>
       <c r="S27" s="9" t="inlineStr"/>
       <c r="T27" s="9" t="inlineStr"/>
-      <c r="U27" s="9" t="inlineStr"/>
+      <c r="U27" s="9" t="inlineStr">
+        <is>
+          <t>Acepción rioplatense = muletilla confirmatoria; "viste" como forma verbal de "ver" es general en todo el español.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -2421,9 +2773,21 @@
       <c r="J28" s="9" t="inlineStr"/>
       <c r="K28" s="9" t="inlineStr"/>
       <c r="L28" s="9" t="inlineStr"/>
-      <c r="M28" s="9" t="inlineStr"/>
-      <c r="N28" s="9" t="inlineStr"/>
-      <c r="O28" s="9" t="inlineStr"/>
+      <c r="M28" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N28" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O28" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P28" s="9" t="inlineStr"/>
       <c r="Q28" s="7">
         <f>IF(OR(J28="",N28=""),"",IF(J28=N28,"sí","no"))</f>
@@ -2482,9 +2846,21 @@
       <c r="J29" s="9" t="inlineStr"/>
       <c r="K29" s="9" t="inlineStr"/>
       <c r="L29" s="9" t="inlineStr"/>
-      <c r="M29" s="9" t="inlineStr"/>
-      <c r="N29" s="9" t="inlineStr"/>
-      <c r="O29" s="9" t="inlineStr"/>
+      <c r="M29" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N29" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O29" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P29" s="9" t="inlineStr"/>
       <c r="Q29" s="7">
         <f>IF(OR(J29="",N29=""),"",IF(J29=N29,"sí","no"))</f>
@@ -2543,9 +2919,21 @@
       <c r="J30" s="9" t="inlineStr"/>
       <c r="K30" s="9" t="inlineStr"/>
       <c r="L30" s="9" t="inlineStr"/>
-      <c r="M30" s="9" t="inlineStr"/>
-      <c r="N30" s="9" t="inlineStr"/>
-      <c r="O30" s="9" t="inlineStr"/>
+      <c r="M30" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N30" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O30" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P30" s="9" t="inlineStr"/>
       <c r="Q30" s="7">
         <f>IF(OR(J30="",N30=""),"",IF(J30=N30,"sí","no"))</f>
@@ -2604,9 +2992,21 @@
       <c r="J31" s="9" t="inlineStr"/>
       <c r="K31" s="9" t="inlineStr"/>
       <c r="L31" s="9" t="inlineStr"/>
-      <c r="M31" s="9" t="inlineStr"/>
-      <c r="N31" s="9" t="inlineStr"/>
-      <c r="O31" s="9" t="inlineStr"/>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N31" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O31" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P31" s="9" t="inlineStr"/>
       <c r="Q31" s="7">
         <f>IF(OR(J31="",N31=""),"",IF(J31=N31,"sí","no"))</f>
@@ -2665,9 +3065,21 @@
       <c r="J32" s="9" t="inlineStr"/>
       <c r="K32" s="9" t="inlineStr"/>
       <c r="L32" s="9" t="inlineStr"/>
-      <c r="M32" s="9" t="inlineStr"/>
-      <c r="N32" s="9" t="inlineStr"/>
-      <c r="O32" s="9" t="inlineStr"/>
+      <c r="M32" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P32" s="9" t="inlineStr"/>
       <c r="Q32" s="7">
         <f>IF(OR(J32="",N32=""),"",IF(J32=N32,"sí","no"))</f>
@@ -2726,9 +3138,21 @@
       <c r="J33" s="9" t="inlineStr"/>
       <c r="K33" s="9" t="inlineStr"/>
       <c r="L33" s="9" t="inlineStr"/>
-      <c r="M33" s="9" t="inlineStr"/>
-      <c r="N33" s="9" t="inlineStr"/>
-      <c r="O33" s="9" t="inlineStr"/>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N33" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O33" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P33" s="9" t="inlineStr"/>
       <c r="Q33" s="7">
         <f>IF(OR(J33="",N33=""),"",IF(J33=N33,"sí","no"))</f>
@@ -2740,7 +3164,11 @@
       </c>
       <c r="S33" s="9" t="inlineStr"/>
       <c r="T33" s="9" t="inlineStr"/>
-      <c r="U33" s="9" t="inlineStr"/>
+      <c r="U33" s="9" t="inlineStr">
+        <is>
+          <t>Ni A ni B reflejan claramente el sentido rioplatense de referencia (inhábil en juegos/deportes); ambos suenan al sentido literal. Revisar con Tomás.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -2787,9 +3215,21 @@
       <c r="J34" s="9" t="inlineStr"/>
       <c r="K34" s="9" t="inlineStr"/>
       <c r="L34" s="9" t="inlineStr"/>
-      <c r="M34" s="9" t="inlineStr"/>
-      <c r="N34" s="9" t="inlineStr"/>
-      <c r="O34" s="9" t="inlineStr"/>
+      <c r="M34" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N34" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O34" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P34" s="9" t="inlineStr"/>
       <c r="Q34" s="7">
         <f>IF(OR(J34="",N34=""),"",IF(J34=N34,"sí","no"))</f>
@@ -2848,9 +3288,21 @@
       <c r="J35" s="9" t="inlineStr"/>
       <c r="K35" s="9" t="inlineStr"/>
       <c r="L35" s="9" t="inlineStr"/>
-      <c r="M35" s="9" t="inlineStr"/>
-      <c r="N35" s="9" t="inlineStr"/>
-      <c r="O35" s="9" t="inlineStr"/>
+      <c r="M35" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N35" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P35" s="9" t="inlineStr"/>
       <c r="Q35" s="7">
         <f>IF(OR(J35="",N35=""),"",IF(J35=N35,"sí","no"))</f>
@@ -2909,9 +3361,21 @@
       <c r="J36" s="9" t="inlineStr"/>
       <c r="K36" s="9" t="inlineStr"/>
       <c r="L36" s="9" t="inlineStr"/>
-      <c r="M36" s="9" t="inlineStr"/>
-      <c r="N36" s="9" t="inlineStr"/>
-      <c r="O36" s="9" t="inlineStr"/>
+      <c r="M36" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N36" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O36" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P36" s="9" t="inlineStr"/>
       <c r="Q36" s="7">
         <f>IF(OR(J36="",N36=""),"",IF(J36=N36,"sí","no"))</f>
@@ -2970,9 +3434,21 @@
       <c r="J37" s="9" t="inlineStr"/>
       <c r="K37" s="9" t="inlineStr"/>
       <c r="L37" s="9" t="inlineStr"/>
-      <c r="M37" s="9" t="inlineStr"/>
-      <c r="N37" s="9" t="inlineStr"/>
-      <c r="O37" s="9" t="inlineStr"/>
+      <c r="M37" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N37" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O37" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P37" s="9" t="inlineStr"/>
       <c r="Q37" s="7">
         <f>IF(OR(J37="",N37=""),"",IF(J37=N37,"sí","no"))</f>
@@ -3031,9 +3507,21 @@
       <c r="J38" s="9" t="inlineStr"/>
       <c r="K38" s="9" t="inlineStr"/>
       <c r="L38" s="9" t="inlineStr"/>
-      <c r="M38" s="9" t="inlineStr"/>
-      <c r="N38" s="9" t="inlineStr"/>
-      <c r="O38" s="9" t="inlineStr"/>
+      <c r="M38" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N38" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O38" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P38" s="9" t="inlineStr"/>
       <c r="Q38" s="7">
         <f>IF(OR(J38="",N38=""),"",IF(J38=N38,"sí","no"))</f>
@@ -3045,7 +3533,11 @@
       </c>
       <c r="S38" s="9" t="inlineStr"/>
       <c r="T38" s="9" t="inlineStr"/>
-      <c r="U38" s="9" t="inlineStr"/>
+      <c r="U38" s="9" t="inlineStr">
+        <is>
+          <t>Ni A ni B reflejan claramente el sentido rioplatense de referencia (engañar); ambos suenan al sentido literal. Revisar con Tomás.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
@@ -3092,10 +3584,26 @@
       <c r="J39" s="9" t="inlineStr"/>
       <c r="K39" s="9" t="inlineStr"/>
       <c r="L39" s="9" t="inlineStr"/>
-      <c r="M39" s="9" t="inlineStr"/>
-      <c r="N39" s="9" t="inlineStr"/>
-      <c r="O39" s="9" t="inlineStr"/>
-      <c r="P39" s="9" t="inlineStr"/>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P39" s="9" t="inlineStr">
+        <is>
+          <t>Tortilla de maíz enrollada con relleno, comida típica (Méx.)</t>
+        </is>
+      </c>
       <c r="Q39" s="7">
         <f>IF(OR(J39="",N39=""),"",IF(J39=N39,"sí","no"))</f>
         <v/>
@@ -3153,10 +3661,26 @@
       <c r="J40" s="9" t="inlineStr"/>
       <c r="K40" s="9" t="inlineStr"/>
       <c r="L40" s="9" t="inlineStr"/>
-      <c r="M40" s="9" t="inlineStr"/>
-      <c r="N40" s="9" t="inlineStr"/>
-      <c r="O40" s="9" t="inlineStr"/>
-      <c r="P40" s="9" t="inlineStr"/>
+      <c r="M40" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N40" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O40" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P40" s="9" t="inlineStr">
+        <is>
+          <t>Que tiene bultos o protuberancias (Méx.)</t>
+        </is>
+      </c>
       <c r="Q40" s="7">
         <f>IF(OR(J40="",N40=""),"",IF(J40=N40,"sí","no"))</f>
         <v/>
@@ -3214,9 +3738,21 @@
       <c r="J41" s="9" t="inlineStr"/>
       <c r="K41" s="9" t="inlineStr"/>
       <c r="L41" s="9" t="inlineStr"/>
-      <c r="M41" s="9" t="inlineStr"/>
-      <c r="N41" s="9" t="inlineStr"/>
-      <c r="O41" s="9" t="inlineStr"/>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N41" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O41" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P41" s="9" t="inlineStr"/>
       <c r="Q41" s="7">
         <f>IF(OR(J41="",N41=""),"",IF(J41=N41,"sí","no"))</f>
@@ -3228,7 +3764,11 @@
       </c>
       <c r="S41" s="9" t="inlineStr"/>
       <c r="T41" s="9" t="inlineStr"/>
-      <c r="U41" s="9" t="inlineStr"/>
+      <c r="U41" s="9" t="inlineStr">
+        <is>
+          <t>Al menos 3 acepciones usadas acá: la bebida, jaque mate (ajedrez), y "cabeza" (coloq.).</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="45" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
@@ -3275,8 +3815,16 @@
       <c r="J42" s="9" t="inlineStr"/>
       <c r="K42" s="9" t="inlineStr"/>
       <c r="L42" s="9" t="inlineStr"/>
-      <c r="M42" s="9" t="inlineStr"/>
-      <c r="N42" s="9" t="inlineStr"/>
+      <c r="M42" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N42" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O42" s="9" t="inlineStr"/>
       <c r="P42" s="9" t="inlineStr"/>
       <c r="Q42" s="7">
@@ -3289,7 +3837,11 @@
       </c>
       <c r="S42" s="9" t="inlineStr"/>
       <c r="T42" s="9" t="inlineStr"/>
-      <c r="U42" s="9" t="inlineStr"/>
+      <c r="U42" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos (A ni B) refleja el sentido de referencia (burlarse/tomar el pelo); ambos usan "cargar" en sentido literal de peso. Fragmento sin elegir, revisar con Tomás o posible reemplazo.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -3336,9 +3888,21 @@
       <c r="J43" s="9" t="inlineStr"/>
       <c r="K43" s="9" t="inlineStr"/>
       <c r="L43" s="9" t="inlineStr"/>
-      <c r="M43" s="9" t="inlineStr"/>
-      <c r="N43" s="9" t="inlineStr"/>
-      <c r="O43" s="9" t="inlineStr"/>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N43" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P43" s="9" t="inlineStr"/>
       <c r="Q43" s="7">
         <f>IF(OR(J43="",N43=""),"",IF(J43=N43,"sí","no"))</f>
@@ -3397,9 +3961,21 @@
       <c r="J44" s="9" t="inlineStr"/>
       <c r="K44" s="9" t="inlineStr"/>
       <c r="L44" s="9" t="inlineStr"/>
-      <c r="M44" s="9" t="inlineStr"/>
-      <c r="N44" s="9" t="inlineStr"/>
-      <c r="O44" s="9" t="inlineStr"/>
+      <c r="M44" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N44" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O44" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P44" s="9" t="inlineStr"/>
       <c r="Q44" s="7">
         <f>IF(OR(J44="",N44=""),"",IF(J44=N44,"sí","no"))</f>
@@ -3458,9 +4034,21 @@
       <c r="J45" s="9" t="inlineStr"/>
       <c r="K45" s="9" t="inlineStr"/>
       <c r="L45" s="9" t="inlineStr"/>
-      <c r="M45" s="9" t="inlineStr"/>
-      <c r="N45" s="9" t="inlineStr"/>
-      <c r="O45" s="9" t="inlineStr"/>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O45" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P45" s="9" t="inlineStr"/>
       <c r="Q45" s="7">
         <f>IF(OR(J45="",N45=""),"",IF(J45=N45,"sí","no"))</f>
@@ -3519,9 +4107,21 @@
       <c r="J46" s="9" t="inlineStr"/>
       <c r="K46" s="9" t="inlineStr"/>
       <c r="L46" s="9" t="inlineStr"/>
-      <c r="M46" s="9" t="inlineStr"/>
-      <c r="N46" s="9" t="inlineStr"/>
-      <c r="O46" s="9" t="inlineStr"/>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N46" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O46" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P46" s="9" t="inlineStr"/>
       <c r="Q46" s="7">
         <f>IF(OR(J46="",N46=""),"",IF(J46=N46,"sí","no"))</f>
@@ -3580,9 +4180,21 @@
       <c r="J47" s="9" t="inlineStr"/>
       <c r="K47" s="9" t="inlineStr"/>
       <c r="L47" s="9" t="inlineStr"/>
-      <c r="M47" s="9" t="inlineStr"/>
-      <c r="N47" s="9" t="inlineStr"/>
-      <c r="O47" s="9" t="inlineStr"/>
+      <c r="M47" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N47" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O47" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P47" s="9" t="inlineStr"/>
       <c r="Q47" s="7">
         <f>IF(OR(J47="",N47=""),"",IF(J47=N47,"sí","no"))</f>
@@ -3633,9 +4245,21 @@
       <c r="J48" s="9" t="inlineStr"/>
       <c r="K48" s="9" t="inlineStr"/>
       <c r="L48" s="9" t="inlineStr"/>
-      <c r="M48" s="9" t="inlineStr"/>
-      <c r="N48" s="9" t="inlineStr"/>
-      <c r="O48" s="9" t="inlineStr"/>
+      <c r="M48" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N48" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O48" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P48" s="9" t="inlineStr"/>
       <c r="Q48" s="7">
         <f>IF(OR(J48="",N48=""),"",IF(J48=N48,"sí","no"))</f>
@@ -3694,10 +4318,26 @@
       <c r="J49" s="9" t="inlineStr"/>
       <c r="K49" s="9" t="inlineStr"/>
       <c r="L49" s="9" t="inlineStr"/>
-      <c r="M49" s="9" t="inlineStr"/>
-      <c r="N49" s="9" t="inlineStr"/>
-      <c r="O49" s="9" t="inlineStr"/>
-      <c r="P49" s="9" t="inlineStr"/>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N49" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O49" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P49" s="9" t="inlineStr">
+        <is>
+          <t>Bolera, lugar para jugar al boliche/bowling (Méx.)</t>
+        </is>
+      </c>
       <c r="Q49" s="7">
         <f>IF(OR(J49="",N49=""),"",IF(J49=N49,"sí","no"))</f>
         <v/>
@@ -3755,10 +4395,26 @@
       <c r="J50" s="9" t="inlineStr"/>
       <c r="K50" s="9" t="inlineStr"/>
       <c r="L50" s="9" t="inlineStr"/>
-      <c r="M50" s="9" t="inlineStr"/>
-      <c r="N50" s="9" t="inlineStr"/>
-      <c r="O50" s="9" t="inlineStr"/>
-      <c r="P50" s="9" t="inlineStr"/>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N50" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O50" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P50" s="9" t="inlineStr">
+        <is>
+          <t>Hablar mal de alguien, desacreditarlo (Méx., entre otros)</t>
+        </is>
+      </c>
       <c r="Q50" s="7">
         <f>IF(OR(J50="",N50=""),"",IF(J50=N50,"sí","no"))</f>
         <v/>
@@ -3816,9 +4472,21 @@
       <c r="J51" s="9" t="inlineStr"/>
       <c r="K51" s="9" t="inlineStr"/>
       <c r="L51" s="9" t="inlineStr"/>
-      <c r="M51" s="9" t="inlineStr"/>
-      <c r="N51" s="9" t="inlineStr"/>
-      <c r="O51" s="9" t="inlineStr"/>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N51" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O51" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P51" s="9" t="inlineStr"/>
       <c r="Q51" s="7">
         <f>IF(OR(J51="",N51=""),"",IF(J51=N51,"sí","no"))</f>
@@ -3877,9 +4545,21 @@
       <c r="J52" s="9" t="inlineStr"/>
       <c r="K52" s="9" t="inlineStr"/>
       <c r="L52" s="9" t="inlineStr"/>
-      <c r="M52" s="9" t="inlineStr"/>
-      <c r="N52" s="9" t="inlineStr"/>
-      <c r="O52" s="9" t="inlineStr"/>
+      <c r="M52" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N52" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O52" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P52" s="9" t="inlineStr"/>
       <c r="Q52" s="7">
         <f>IF(OR(J52="",N52=""),"",IF(J52=N52,"sí","no"))</f>
@@ -3938,9 +4618,21 @@
       <c r="J53" s="9" t="inlineStr"/>
       <c r="K53" s="9" t="inlineStr"/>
       <c r="L53" s="9" t="inlineStr"/>
-      <c r="M53" s="9" t="inlineStr"/>
-      <c r="N53" s="9" t="inlineStr"/>
-      <c r="O53" s="9" t="inlineStr"/>
+      <c r="M53" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N53" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O53" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P53" s="9" t="inlineStr"/>
       <c r="Q53" s="7">
         <f>IF(OR(J53="",N53=""),"",IF(J53=N53,"sí","no"))</f>
@@ -3999,9 +4691,21 @@
       <c r="J54" s="9" t="inlineStr"/>
       <c r="K54" s="9" t="inlineStr"/>
       <c r="L54" s="9" t="inlineStr"/>
-      <c r="M54" s="9" t="inlineStr"/>
-      <c r="N54" s="9" t="inlineStr"/>
-      <c r="O54" s="9" t="inlineStr"/>
+      <c r="M54" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N54" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O54" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P54" s="9" t="inlineStr"/>
       <c r="Q54" s="7">
         <f>IF(OR(J54="",N54=""),"",IF(J54=N54,"sí","no"))</f>
@@ -4060,10 +4764,22 @@
       <c r="J55" s="9" t="inlineStr"/>
       <c r="K55" s="9" t="inlineStr"/>
       <c r="L55" s="9" t="inlineStr"/>
-      <c r="M55" s="9" t="inlineStr"/>
-      <c r="N55" s="9" t="inlineStr"/>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N55" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
       <c r="O55" s="9" t="inlineStr"/>
-      <c r="P55" s="9" t="inlineStr"/>
+      <c r="P55" s="9" t="inlineStr">
+        <is>
+          <t>Irse/escapar precipitadamente, o morir (Méx., El Salv.)</t>
+        </is>
+      </c>
       <c r="Q55" s="7">
         <f>IF(OR(J55="",N55=""),"",IF(J55=N55,"sí","no"))</f>
         <v/>
@@ -4074,7 +4790,11 @@
       </c>
       <c r="S55" s="9" t="inlineStr"/>
       <c r="T55" s="9" t="inlineStr"/>
-      <c r="U55" s="9" t="inlineStr"/>
+      <c r="U55" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos refleja con claridad "sacar plata a alguien"; A es ambiguo (posible arma) y B es sobre pelar cables de cobre, literal. Fragmento sin elegir, revisar con Tomás o posible reemplazo.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="75" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
@@ -4121,8 +4841,16 @@
       <c r="J56" s="9" t="inlineStr"/>
       <c r="K56" s="9" t="inlineStr"/>
       <c r="L56" s="9" t="inlineStr"/>
-      <c r="M56" s="9" t="inlineStr"/>
-      <c r="N56" s="9" t="inlineStr"/>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N56" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O56" s="9" t="inlineStr"/>
       <c r="P56" s="9" t="inlineStr"/>
       <c r="Q56" s="7">
@@ -4135,7 +4863,11 @@
       </c>
       <c r="S56" s="9" t="inlineStr"/>
       <c r="T56" s="9" t="inlineStr"/>
-      <c r="U56" s="9" t="inlineStr"/>
+      <c r="U56" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos usa el sentido de referencia (corte de carne); ambos son el sentido figurado de "vacío emocional". Fragmento sin elegir, revisar con Tomás o posible reemplazo.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
@@ -4182,9 +4914,21 @@
       <c r="J57" s="9" t="inlineStr"/>
       <c r="K57" s="9" t="inlineStr"/>
       <c r="L57" s="9" t="inlineStr"/>
-      <c r="M57" s="9" t="inlineStr"/>
-      <c r="N57" s="9" t="inlineStr"/>
-      <c r="O57" s="9" t="inlineStr"/>
+      <c r="M57" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N57" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O57" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P57" s="9" t="inlineStr"/>
       <c r="Q57" s="7">
         <f>IF(OR(J57="",N57=""),"",IF(J57=N57,"sí","no"))</f>
@@ -4243,9 +4987,21 @@
       <c r="J58" s="9" t="inlineStr"/>
       <c r="K58" s="9" t="inlineStr"/>
       <c r="L58" s="9" t="inlineStr"/>
-      <c r="M58" s="9" t="inlineStr"/>
-      <c r="N58" s="9" t="inlineStr"/>
-      <c r="O58" s="9" t="inlineStr"/>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N58" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O58" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P58" s="9" t="inlineStr"/>
       <c r="Q58" s="7">
         <f>IF(OR(J58="",N58=""),"",IF(J58=N58,"sí","no"))</f>
@@ -4304,8 +5060,16 @@
       <c r="J59" s="9" t="inlineStr"/>
       <c r="K59" s="9" t="inlineStr"/>
       <c r="L59" s="9" t="inlineStr"/>
-      <c r="M59" s="9" t="inlineStr"/>
-      <c r="N59" s="9" t="inlineStr"/>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N59" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O59" s="9" t="inlineStr"/>
       <c r="P59" s="9" t="inlineStr"/>
       <c r="Q59" s="7">
@@ -4318,7 +5082,11 @@
       </c>
       <c r="S59" s="9" t="inlineStr"/>
       <c r="T59" s="9" t="inlineStr"/>
-      <c r="U59" s="9" t="inlineStr"/>
+      <c r="U59" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos refleja el sentido de referencia (aguantar/soportar); ambos usan "fumar" literalmente (cigarrillo/porro). Fragmento sin elegir, revisar con Tomás o posible reemplazo.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="45" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
@@ -4365,9 +5133,21 @@
       <c r="J60" s="9" t="inlineStr"/>
       <c r="K60" s="9" t="inlineStr"/>
       <c r="L60" s="9" t="inlineStr"/>
-      <c r="M60" s="9" t="inlineStr"/>
-      <c r="N60" s="9" t="inlineStr"/>
-      <c r="O60" s="9" t="inlineStr"/>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N60" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O60" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P60" s="9" t="inlineStr"/>
       <c r="Q60" s="7">
         <f>IF(OR(J60="",N60=""),"",IF(J60=N60,"sí","no"))</f>
@@ -4426,9 +5206,21 @@
       <c r="J61" s="9" t="inlineStr"/>
       <c r="K61" s="9" t="inlineStr"/>
       <c r="L61" s="9" t="inlineStr"/>
-      <c r="M61" s="9" t="inlineStr"/>
-      <c r="N61" s="9" t="inlineStr"/>
-      <c r="O61" s="9" t="inlineStr"/>
+      <c r="M61" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N61" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O61" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P61" s="9" t="inlineStr"/>
       <c r="Q61" s="7">
         <f>IF(OR(J61="",N61=""),"",IF(J61=N61,"sí","no"))</f>
@@ -4487,9 +5279,21 @@
       <c r="J62" s="9" t="inlineStr"/>
       <c r="K62" s="9" t="inlineStr"/>
       <c r="L62" s="9" t="inlineStr"/>
-      <c r="M62" s="9" t="inlineStr"/>
-      <c r="N62" s="9" t="inlineStr"/>
-      <c r="O62" s="9" t="inlineStr"/>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N62" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O62" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P62" s="9" t="inlineStr"/>
       <c r="Q62" s="7">
         <f>IF(OR(J62="",N62=""),"",IF(J62=N62,"sí","no"))</f>
@@ -4548,9 +5352,21 @@
       <c r="J63" s="9" t="inlineStr"/>
       <c r="K63" s="9" t="inlineStr"/>
       <c r="L63" s="9" t="inlineStr"/>
-      <c r="M63" s="9" t="inlineStr"/>
-      <c r="N63" s="9" t="inlineStr"/>
-      <c r="O63" s="9" t="inlineStr"/>
+      <c r="M63" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N63" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O63" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P63" s="9" t="inlineStr"/>
       <c r="Q63" s="7">
         <f>IF(OR(J63="",N63=""),"",IF(J63=N63,"sí","no"))</f>
@@ -4609,9 +5425,21 @@
       <c r="J64" s="9" t="inlineStr"/>
       <c r="K64" s="9" t="inlineStr"/>
       <c r="L64" s="9" t="inlineStr"/>
-      <c r="M64" s="9" t="inlineStr"/>
-      <c r="N64" s="9" t="inlineStr"/>
-      <c r="O64" s="9" t="inlineStr"/>
+      <c r="M64" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N64" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O64" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P64" s="9" t="inlineStr"/>
       <c r="Q64" s="7">
         <f>IF(OR(J64="",N64=""),"",IF(J64=N64,"sí","no"))</f>
@@ -4623,7 +5451,11 @@
       </c>
       <c r="S64" s="9" t="inlineStr"/>
       <c r="T64" s="9" t="inlineStr"/>
-      <c r="U64" s="9" t="inlineStr"/>
+      <c r="U64" s="9" t="inlineStr">
+        <is>
+          <t>Nombre del género musical, préstamo del inglés usado igual en todos los dialectos; no tiene carga rioplatense.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="45" customHeight="1">
       <c r="A65" s="7" t="inlineStr">
@@ -4670,9 +5502,21 @@
       <c r="J65" s="9" t="inlineStr"/>
       <c r="K65" s="9" t="inlineStr"/>
       <c r="L65" s="9" t="inlineStr"/>
-      <c r="M65" s="9" t="inlineStr"/>
-      <c r="N65" s="9" t="inlineStr"/>
-      <c r="O65" s="9" t="inlineStr"/>
+      <c r="M65" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N65" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O65" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P65" s="9" t="inlineStr"/>
       <c r="Q65" s="7">
         <f>IF(OR(J65="",N65=""),"",IF(J65=N65,"sí","no"))</f>
@@ -4731,9 +5575,21 @@
       <c r="J66" s="9" t="inlineStr"/>
       <c r="K66" s="9" t="inlineStr"/>
       <c r="L66" s="9" t="inlineStr"/>
-      <c r="M66" s="9" t="inlineStr"/>
-      <c r="N66" s="9" t="inlineStr"/>
-      <c r="O66" s="9" t="inlineStr"/>
+      <c r="M66" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N66" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O66" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P66" s="9" t="inlineStr"/>
       <c r="Q66" s="7">
         <f>IF(OR(J66="",N66=""),"",IF(J66=N66,"sí","no"))</f>
@@ -4792,9 +5648,21 @@
       <c r="J67" s="9" t="inlineStr"/>
       <c r="K67" s="9" t="inlineStr"/>
       <c r="L67" s="9" t="inlineStr"/>
-      <c r="M67" s="9" t="inlineStr"/>
-      <c r="N67" s="9" t="inlineStr"/>
-      <c r="O67" s="9" t="inlineStr"/>
+      <c r="M67" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N67" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O67" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P67" s="9" t="inlineStr"/>
       <c r="Q67" s="7">
         <f>IF(OR(J67="",N67=""),"",IF(J67=N67,"sí","no"))</f>
@@ -4853,8 +5721,16 @@
       <c r="J68" s="9" t="inlineStr"/>
       <c r="K68" s="9" t="inlineStr"/>
       <c r="L68" s="9" t="inlineStr"/>
-      <c r="M68" s="9" t="inlineStr"/>
-      <c r="N68" s="9" t="inlineStr"/>
+      <c r="M68" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N68" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O68" s="9" t="inlineStr"/>
       <c r="P68" s="9" t="inlineStr"/>
       <c r="Q68" s="7">
@@ -4867,7 +5743,11 @@
       </c>
       <c r="S68" s="9" t="inlineStr"/>
       <c r="T68" s="9" t="inlineStr"/>
-      <c r="U68" s="9" t="inlineStr"/>
+      <c r="U68" s="9" t="inlineStr">
+        <is>
+          <t>Ni A ni B reflejan "situación/persona divertida" con claridad (A es el modismo "dar gato por liebre" = engañar; B es un modismo de recaudación). Candidato a reemplazo: re-correr pipeline/stage03b_contextos.py apuntado a este término con tope más alto.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="7" t="inlineStr">
@@ -4914,10 +5794,22 @@
       <c r="J69" s="9" t="inlineStr"/>
       <c r="K69" s="9" t="inlineStr"/>
       <c r="L69" s="9" t="inlineStr"/>
-      <c r="M69" s="9" t="inlineStr"/>
-      <c r="N69" s="9" t="inlineStr"/>
+      <c r="M69" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N69" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
       <c r="O69" s="9" t="inlineStr"/>
-      <c r="P69" s="9" t="inlineStr"/>
+      <c r="P69" s="9" t="inlineStr">
+        <is>
+          <t>Desacreditar (El Salv. y Méx.)</t>
+        </is>
+      </c>
       <c r="Q69" s="7">
         <f>IF(OR(J69="",N69=""),"",IF(J69=N69,"sí","no"))</f>
         <v/>
@@ -4928,7 +5820,11 @@
       </c>
       <c r="S69" s="9" t="inlineStr"/>
       <c r="T69" s="9" t="inlineStr"/>
-      <c r="U69" s="9" t="inlineStr"/>
+      <c r="U69" s="9" t="inlineStr">
+        <is>
+          <t>B suena a "fumar algo" más que a "delatar/burlar", que es la acepción de referencia. Candidato a reemplazo, re-correr el pipeline para este término.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="7" t="inlineStr">
@@ -4975,9 +5871,21 @@
       <c r="J70" s="9" t="inlineStr"/>
       <c r="K70" s="9" t="inlineStr"/>
       <c r="L70" s="9" t="inlineStr"/>
-      <c r="M70" s="9" t="inlineStr"/>
-      <c r="N70" s="9" t="inlineStr"/>
-      <c r="O70" s="9" t="inlineStr"/>
+      <c r="M70" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N70" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O70" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P70" s="9" t="inlineStr"/>
       <c r="Q70" s="7">
         <f>IF(OR(J70="",N70=""),"",IF(J70=N70,"sí","no"))</f>
@@ -5036,9 +5944,21 @@
       <c r="J71" s="9" t="inlineStr"/>
       <c r="K71" s="9" t="inlineStr"/>
       <c r="L71" s="9" t="inlineStr"/>
-      <c r="M71" s="9" t="inlineStr"/>
-      <c r="N71" s="9" t="inlineStr"/>
-      <c r="O71" s="9" t="inlineStr"/>
+      <c r="M71" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N71" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O71" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P71" s="9" t="inlineStr"/>
       <c r="Q71" s="7">
         <f>IF(OR(J71="",N71=""),"",IF(J71=N71,"sí","no"))</f>
@@ -5097,9 +6017,21 @@
       <c r="J72" s="9" t="inlineStr"/>
       <c r="K72" s="9" t="inlineStr"/>
       <c r="L72" s="9" t="inlineStr"/>
-      <c r="M72" s="9" t="inlineStr"/>
-      <c r="N72" s="9" t="inlineStr"/>
-      <c r="O72" s="9" t="inlineStr"/>
+      <c r="M72" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N72" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O72" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P72" s="9" t="inlineStr"/>
       <c r="Q72" s="7">
         <f>IF(OR(J72="",N72=""),"",IF(J72=N72,"sí","no"))</f>
@@ -5158,8 +6090,16 @@
       <c r="J73" s="9" t="inlineStr"/>
       <c r="K73" s="9" t="inlineStr"/>
       <c r="L73" s="9" t="inlineStr"/>
-      <c r="M73" s="9" t="inlineStr"/>
-      <c r="N73" s="9" t="inlineStr"/>
+      <c r="M73" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N73" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O73" s="9" t="inlineStr"/>
       <c r="P73" s="9" t="inlineStr"/>
       <c r="Q73" s="7">
@@ -5172,7 +6112,11 @@
       </c>
       <c r="S73" s="9" t="inlineStr"/>
       <c r="T73" s="9" t="inlineStr"/>
-      <c r="U73" s="9" t="inlineStr"/>
+      <c r="U73" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos usa claramente el sentido "caro/costoso". Candidato a reemplazo, re-correr el pipeline para este término.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="45" customHeight="1">
       <c r="A74" s="7" t="inlineStr">
@@ -5219,9 +6163,21 @@
       <c r="J74" s="9" t="inlineStr"/>
       <c r="K74" s="9" t="inlineStr"/>
       <c r="L74" s="9" t="inlineStr"/>
-      <c r="M74" s="9" t="inlineStr"/>
-      <c r="N74" s="9" t="inlineStr"/>
-      <c r="O74" s="9" t="inlineStr"/>
+      <c r="M74" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N74" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O74" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P74" s="9" t="inlineStr"/>
       <c r="Q74" s="7">
         <f>IF(OR(J74="",N74=""),"",IF(J74=N74,"sí","no"))</f>
@@ -5280,9 +6236,21 @@
       <c r="J75" s="9" t="inlineStr"/>
       <c r="K75" s="9" t="inlineStr"/>
       <c r="L75" s="9" t="inlineStr"/>
-      <c r="M75" s="9" t="inlineStr"/>
-      <c r="N75" s="9" t="inlineStr"/>
-      <c r="O75" s="9" t="inlineStr"/>
+      <c r="M75" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N75" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O75" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P75" s="9" t="inlineStr"/>
       <c r="Q75" s="7">
         <f>IF(OR(J75="",N75=""),"",IF(J75=N75,"sí","no"))</f>
@@ -5333,9 +6301,21 @@
       <c r="J76" s="9" t="inlineStr"/>
       <c r="K76" s="9" t="inlineStr"/>
       <c r="L76" s="9" t="inlineStr"/>
-      <c r="M76" s="9" t="inlineStr"/>
-      <c r="N76" s="9" t="inlineStr"/>
-      <c r="O76" s="9" t="inlineStr"/>
+      <c r="M76" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N76" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O76" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P76" s="9" t="inlineStr"/>
       <c r="Q76" s="7">
         <f>IF(OR(J76="",N76=""),"",IF(J76=N76,"sí","no"))</f>
@@ -5394,10 +6374,22 @@
       <c r="J77" s="9" t="inlineStr"/>
       <c r="K77" s="9" t="inlineStr"/>
       <c r="L77" s="9" t="inlineStr"/>
-      <c r="M77" s="9" t="inlineStr"/>
-      <c r="N77" s="9" t="inlineStr"/>
+      <c r="M77" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N77" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
       <c r="O77" s="9" t="inlineStr"/>
-      <c r="P77" s="9" t="inlineStr"/>
+      <c r="P77" s="9" t="inlineStr">
+        <is>
+          <t>Moneda de cinco pesetas, ya desaparecida (Esp.)</t>
+        </is>
+      </c>
       <c r="Q77" s="7">
         <f>IF(OR(J77="",N77=""),"",IF(J77=N77,"sí","no"))</f>
         <v/>
@@ -5408,7 +6400,11 @@
       </c>
       <c r="S77" s="9" t="inlineStr"/>
       <c r="T77" s="9" t="inlineStr"/>
-      <c r="U77" s="9" t="inlineStr"/>
+      <c r="U77" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos usa el sentido "drogado"; ambos parecen literales/figurados distintos. Candidato a reemplazo, re-correr el pipeline para este término.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="45" customHeight="1">
       <c r="A78" s="7" t="inlineStr">
@@ -5455,9 +6451,21 @@
       <c r="J78" s="9" t="inlineStr"/>
       <c r="K78" s="9" t="inlineStr"/>
       <c r="L78" s="9" t="inlineStr"/>
-      <c r="M78" s="9" t="inlineStr"/>
-      <c r="N78" s="9" t="inlineStr"/>
-      <c r="O78" s="9" t="inlineStr"/>
+      <c r="M78" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N78" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O78" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P78" s="9" t="inlineStr"/>
       <c r="Q78" s="7">
         <f>IF(OR(J78="",N78=""),"",IF(J78=N78,"sí","no"))</f>
@@ -5516,9 +6524,21 @@
       <c r="J79" s="9" t="inlineStr"/>
       <c r="K79" s="9" t="inlineStr"/>
       <c r="L79" s="9" t="inlineStr"/>
-      <c r="M79" s="9" t="inlineStr"/>
-      <c r="N79" s="9" t="inlineStr"/>
-      <c r="O79" s="9" t="inlineStr"/>
+      <c r="M79" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N79" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O79" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P79" s="9" t="inlineStr"/>
       <c r="Q79" s="7">
         <f>IF(OR(J79="",N79=""),"",IF(J79=N79,"sí","no"))</f>
@@ -5577,9 +6597,21 @@
       <c r="J80" s="9" t="inlineStr"/>
       <c r="K80" s="9" t="inlineStr"/>
       <c r="L80" s="9" t="inlineStr"/>
-      <c r="M80" s="9" t="inlineStr"/>
-      <c r="N80" s="9" t="inlineStr"/>
-      <c r="O80" s="9" t="inlineStr"/>
+      <c r="M80" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N80" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O80" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P80" s="9" t="inlineStr"/>
       <c r="Q80" s="7">
         <f>IF(OR(J80="",N80=""),"",IF(J80=N80,"sí","no"))</f>
@@ -5638,8 +6670,16 @@
       <c r="J81" s="9" t="inlineStr"/>
       <c r="K81" s="9" t="inlineStr"/>
       <c r="L81" s="9" t="inlineStr"/>
-      <c r="M81" s="9" t="inlineStr"/>
-      <c r="N81" s="9" t="inlineStr"/>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N81" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O81" s="9" t="inlineStr"/>
       <c r="P81" s="9" t="inlineStr"/>
       <c r="Q81" s="7">
@@ -5652,7 +6692,11 @@
       </c>
       <c r="S81" s="9" t="inlineStr"/>
       <c r="T81" s="9" t="inlineStr"/>
-      <c r="U81" s="9" t="inlineStr"/>
+      <c r="U81" s="9" t="inlineStr">
+        <is>
+          <t>B usa "bate" (el objeto/palo), no el verbo "batir" en sentido de delatar. Candidato a revisar "El Ciruja" (tango clásico con mucho lunfardo) como fuente alternativa, o re-correr el pipeline.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="45" customHeight="1">
       <c r="A82" s="7" t="inlineStr">
@@ -5699,9 +6743,21 @@
       <c r="J82" s="9" t="inlineStr"/>
       <c r="K82" s="9" t="inlineStr"/>
       <c r="L82" s="9" t="inlineStr"/>
-      <c r="M82" s="9" t="inlineStr"/>
-      <c r="N82" s="9" t="inlineStr"/>
-      <c r="O82" s="9" t="inlineStr"/>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N82" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O82" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P82" s="9" t="inlineStr"/>
       <c r="Q82" s="7">
         <f>IF(OR(J82="",N82=""),"",IF(J82=N82,"sí","no"))</f>
@@ -5760,9 +6816,21 @@
       <c r="J83" s="9" t="inlineStr"/>
       <c r="K83" s="9" t="inlineStr"/>
       <c r="L83" s="9" t="inlineStr"/>
-      <c r="M83" s="9" t="inlineStr"/>
-      <c r="N83" s="9" t="inlineStr"/>
-      <c r="O83" s="9" t="inlineStr"/>
+      <c r="M83" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N83" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O83" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P83" s="9" t="inlineStr"/>
       <c r="Q83" s="7">
         <f>IF(OR(J83="",N83=""),"",IF(J83=N83,"sí","no"))</f>
@@ -5821,9 +6889,21 @@
       <c r="J84" s="9" t="inlineStr"/>
       <c r="K84" s="9" t="inlineStr"/>
       <c r="L84" s="9" t="inlineStr"/>
-      <c r="M84" s="9" t="inlineStr"/>
-      <c r="N84" s="9" t="inlineStr"/>
-      <c r="O84" s="9" t="inlineStr"/>
+      <c r="M84" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N84" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O84" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P84" s="9" t="inlineStr"/>
       <c r="Q84" s="7">
         <f>IF(OR(J84="",N84=""),"",IF(J84=N84,"sí","no"))</f>
@@ -5882,8 +6962,16 @@
       <c r="J85" s="9" t="inlineStr"/>
       <c r="K85" s="9" t="inlineStr"/>
       <c r="L85" s="9" t="inlineStr"/>
-      <c r="M85" s="9" t="inlineStr"/>
-      <c r="N85" s="9" t="inlineStr"/>
+      <c r="M85" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N85" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O85" s="9" t="inlineStr"/>
       <c r="P85" s="9" t="inlineStr"/>
       <c r="Q85" s="7">
@@ -5896,7 +6984,11 @@
       </c>
       <c r="S85" s="9" t="inlineStr"/>
       <c r="T85" s="9" t="inlineStr"/>
-      <c r="U85" s="9" t="inlineStr"/>
+      <c r="U85" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos refleja "emborracharse hasta vomitar"; B es sobre un paso de baile. Candidato a reemplazo, re-correr el pipeline para este término.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="60" customHeight="1">
       <c r="A86" s="7" t="inlineStr">
@@ -5943,9 +7035,21 @@
       <c r="J86" s="9" t="inlineStr"/>
       <c r="K86" s="9" t="inlineStr"/>
       <c r="L86" s="9" t="inlineStr"/>
-      <c r="M86" s="9" t="inlineStr"/>
-      <c r="N86" s="9" t="inlineStr"/>
-      <c r="O86" s="9" t="inlineStr"/>
+      <c r="M86" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N86" s="9" t="inlineStr">
+        <is>
+          <t>espanol_general</t>
+        </is>
+      </c>
+      <c r="O86" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P86" s="9" t="inlineStr"/>
       <c r="Q86" s="7">
         <f>IF(OR(J86="",N86=""),"",IF(J86=N86,"sí","no"))</f>
@@ -6004,10 +7108,26 @@
       <c r="J87" s="9" t="inlineStr"/>
       <c r="K87" s="9" t="inlineStr"/>
       <c r="L87" s="9" t="inlineStr"/>
-      <c r="M87" s="9" t="inlineStr"/>
-      <c r="N87" s="9" t="inlineStr"/>
-      <c r="O87" s="9" t="inlineStr"/>
-      <c r="P87" s="9" t="inlineStr"/>
+      <c r="M87" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N87" s="9" t="inlineStr">
+        <is>
+          <t>falso_amigo</t>
+        </is>
+      </c>
+      <c r="O87" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P87" s="9" t="inlineStr">
+        <is>
+          <t>Persona nacida en Madrid (coloq., Esp.)</t>
+        </is>
+      </c>
       <c r="Q87" s="7">
         <f>IF(OR(J87="",N87=""),"",IF(J87=N87,"sí","no"))</f>
         <v/>
@@ -6065,9 +7185,21 @@
       <c r="J88" s="9" t="inlineStr"/>
       <c r="K88" s="9" t="inlineStr"/>
       <c r="L88" s="9" t="inlineStr"/>
-      <c r="M88" s="9" t="inlineStr"/>
-      <c r="N88" s="9" t="inlineStr"/>
-      <c r="O88" s="9" t="inlineStr"/>
+      <c r="M88" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N88" s="9" t="inlineStr">
+        <is>
+          <t>lunfardo_sin_homonimo</t>
+        </is>
+      </c>
+      <c r="O88" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P88" s="9" t="inlineStr"/>
       <c r="Q88" s="7">
         <f>IF(OR(J88="",N88=""),"",IF(J88=N88,"sí","no"))</f>
@@ -6126,9 +7258,21 @@
       <c r="J89" s="9" t="inlineStr"/>
       <c r="K89" s="9" t="inlineStr"/>
       <c r="L89" s="9" t="inlineStr"/>
-      <c r="M89" s="9" t="inlineStr"/>
-      <c r="N89" s="9" t="inlineStr"/>
-      <c r="O89" s="9" t="inlineStr"/>
+      <c r="M89" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N89" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O89" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="P89" s="9" t="inlineStr"/>
       <c r="Q89" s="7">
         <f>IF(OR(J89="",N89=""),"",IF(J89=N89,"sí","no"))</f>
@@ -6187,9 +7331,21 @@
       <c r="J90" s="9" t="inlineStr"/>
       <c r="K90" s="9" t="inlineStr"/>
       <c r="L90" s="9" t="inlineStr"/>
-      <c r="M90" s="9" t="inlineStr"/>
-      <c r="N90" s="9" t="inlineStr"/>
-      <c r="O90" s="9" t="inlineStr"/>
+      <c r="M90" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N90" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
+      <c r="O90" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="P90" s="9" t="inlineStr"/>
       <c r="Q90" s="7">
         <f>IF(OR(J90="",N90=""),"",IF(J90=N90,"sí","no"))</f>
@@ -6248,8 +7404,16 @@
       <c r="J91" s="9" t="inlineStr"/>
       <c r="K91" s="9" t="inlineStr"/>
       <c r="L91" s="9" t="inlineStr"/>
-      <c r="M91" s="9" t="inlineStr"/>
-      <c r="N91" s="9" t="inlineStr"/>
+      <c r="M91" s="9" t="inlineStr">
+        <is>
+          <t>Valentín Garfi</t>
+        </is>
+      </c>
+      <c r="N91" s="9" t="inlineStr">
+        <is>
+          <t>polisemico_interno</t>
+        </is>
+      </c>
       <c r="O91" s="9" t="inlineStr"/>
       <c r="P91" s="9" t="inlineStr"/>
       <c r="Q91" s="7">
@@ -6262,7 +7426,11 @@
       </c>
       <c r="S91" s="9" t="inlineStr"/>
       <c r="T91" s="9" t="inlineStr"/>
-      <c r="U91" s="9" t="inlineStr"/>
+      <c r="U91" s="9" t="inlineStr">
+        <is>
+          <t>Ninguno de los dos fragmentos usa el sentido "paquete de cigarrillos"; ambos son el participio literal de "atar". Candidato a reemplazo, re-correr el pipeline para este término.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U91"/>

</xml_diff>